<commit_message>
Rebuild Excel with full Solver step-by-step configuration
Each sheet now includes a detailed "CONFIGURAÇÃO DO SOLVER — PASSO A PASSO"
section with exact cell references for: Objective cell, Variable cells,
all constraints (LHS cell, operator, RHS cell), method (Simplex LP),
and numbered steps 1-8 matching the Excel Solver dialog.

https://claude.ai/code/session_011k96wFEvzHdLWjiCrVuMUh
</commit_message>
<xml_diff>
--- a/QUIZZES_3_e_4_Samuel.xlsx
+++ b/QUIZZES_3_e_4_Samuel.xlsx
@@ -21,7 +21,7 @@
     <numFmt numFmtId="164" formatCode="$#,##0"/>
     <numFmt numFmtId="165" formatCode="$#,##0.00"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -33,11 +33,6 @@
       <name val="Arial"/>
       <b val="1"/>
       <sz val="14"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <sz val="12"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -67,10 +62,27 @@
     </font>
     <font>
       <name val="Arial"/>
+      <b val="1"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00000000"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FF0000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -80,25 +92,26 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="004472C4"/>
-        <bgColor rgb="004472C4"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00D9D9D9"/>
-        <bgColor rgb="00D9D9D9"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFFF00"/>
-        <bgColor rgb="00FFFF00"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFCC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00E2EFDA"/>
-        <bgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
   </fills>
@@ -134,59 +147,72 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="1" fontId="6" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="6" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="2" fillId="4" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="1" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="1" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="8" fillId="4" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="7" fillId="4" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -278,7 +304,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Análise de Sensibilidade: Capacidade vs Custo Total</a:t>
+              <a:t>Análise de Sensibilidade: Capacidade Máxima por Arco vs Custo Total</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -292,7 +318,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Quiz 4 - Distribuição'!B101</f>
+              <f>'Quiz 4 - Distribuição'!B123</f>
             </strRef>
           </tx>
           <spPr>
@@ -310,12 +336,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Quiz 4 - Distribuição'!$A$102:$A$112</f>
+              <f>'Quiz 4 - Distribuição'!$A$124:$A$134</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Quiz 4 - Distribuição'!$B$102:$B$112</f>
+              <f>'Quiz 4 - Distribuição'!$B$124:$B$134</f>
             </numRef>
           </val>
         </ser>
@@ -337,7 +363,7 @@
                   <a:defRPr/>
                 </a:pPr>
                 <a:r>
-                  <a:t>Capacidade Máxima por Arco</a:t>
+                  <a:t>Capacidade Máxima por Arco (veículos)</a:t>
                 </a:r>
               </a:p>
             </rich>
@@ -390,10 +416,10 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>129</row>
+      <row>153</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="9000000" cy="5400000"/>
+    <ext cx="10080000" cy="5760000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="1" name="Chart 1"/>
@@ -700,23 +726,24 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H92"/>
+  <dimension ref="A1:H109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>QUIZ 3 — Localização de Armazéns (MILP)</t>
+          <t>QUIZ 3 — Localização de Armazéns (Programação Linear Inteira Mista)</t>
         </is>
       </c>
     </row>
@@ -737,7 +764,7 @@
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>Custos Unitários (Produção + Transporte)</t>
+          <t>Custos Unitários de Produção + Transporte ($/unidade)</t>
         </is>
       </c>
     </row>
@@ -889,7 +916,7 @@
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>Demandas Semanais</t>
+          <t>Demandas Semanais por Região</t>
         </is>
       </c>
     </row>
@@ -938,7 +965,7 @@
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>Capacidade por armazém:</t>
+          <t>Capacidade máx. por armazém:</t>
         </is>
       </c>
       <c r="B25" s="9" t="n">
@@ -948,7 +975,7 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>2. VARIÁVEIS DE DECISÃO</t>
+          <t>2. VARIÁVEIS DE DECISÃO (células que o Solver altera)</t>
         </is>
       </c>
       <c r="B27" s="3" t="n"/>
@@ -962,29 +989,29 @@
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>Variáveis Binárias (y_i = 1 se armazém i é aberto)</t>
+          <t>y_i — Abrir armazém? (0 ou 1) → VARIÁVEIS BINÁRIAS</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t>NY</t>
+          <t>y_NY</t>
         </is>
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>LA</t>
+          <t>y_LA</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>Chicago</t>
+          <t>y_Chicago</t>
         </is>
       </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
-          <t>Atlanta</t>
+          <t>y_Atlanta</t>
         </is>
       </c>
     </row>
@@ -1005,14 +1032,14 @@
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
         <is>
-          <t>Variáveis de Envio x_ij (unidades armazém → região)</t>
+          <t>x_ij — Unidades enviadas de armazém i → região j → VARIÁVEIS CONTÍNUAS</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="5" t="inlineStr">
         <is>
-          <t>Armazém</t>
+          <t>x_ij</t>
         </is>
       </c>
       <c r="B34" s="5" t="inlineStr">
@@ -1032,105 +1059,105 @@
       </c>
       <c r="E34" s="5" t="inlineStr">
         <is>
-          <t>Total Enviado</t>
+          <t>Total Enviado (LHS cap.)</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="11" t="inlineStr">
+      <c r="A35" s="5" t="inlineStr">
         <is>
           <t>NY</t>
         </is>
       </c>
-      <c r="B35" s="12" t="n">
+      <c r="B35" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="C35" s="12" t="n">
+      <c r="C35" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="D35" s="12" t="n">
+      <c r="D35" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="E35" s="13">
+      <c r="E35" s="12">
         <f>SUM(B35:D35)</f>
         <v/>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="11" t="inlineStr">
+      <c r="A36" s="5" t="inlineStr">
         <is>
           <t>LA</t>
         </is>
       </c>
-      <c r="B36" s="12" t="n">
+      <c r="B36" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="C36" s="12" t="n">
+      <c r="C36" s="11" t="n">
         <v>8000</v>
       </c>
-      <c r="D36" s="12" t="n">
+      <c r="D36" s="11" t="n">
         <v>7000</v>
       </c>
-      <c r="E36" s="13">
+      <c r="E36" s="12">
         <f>SUM(B36:D36)</f>
         <v/>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="11" t="inlineStr">
+      <c r="A37" s="5" t="inlineStr">
         <is>
           <t>Chicago</t>
         </is>
       </c>
-      <c r="B37" s="12" t="n">
+      <c r="B37" s="11" t="n">
         <v>8000</v>
       </c>
-      <c r="C37" s="12" t="n">
+      <c r="C37" s="11" t="n">
         <v>1000</v>
       </c>
-      <c r="D37" s="12" t="n">
+      <c r="D37" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="E37" s="13">
+      <c r="E37" s="12">
         <f>SUM(B37:D37)</f>
         <v/>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="11" t="inlineStr">
+      <c r="A38" s="5" t="inlineStr">
         <is>
           <t>Atlanta</t>
         </is>
       </c>
-      <c r="B38" s="12" t="n">
+      <c r="B38" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="C38" s="12" t="n">
+      <c r="C38" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="D38" s="12" t="n">
+      <c r="D38" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="E38" s="13">
+      <c r="E38" s="12">
         <f>SUM(B38:D38)</f>
         <v/>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="11" t="inlineStr">
-        <is>
-          <t>Total Recebido</t>
-        </is>
-      </c>
-      <c r="B39" s="13">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>Total Recebido (LHS dem.)</t>
+        </is>
+      </c>
+      <c r="B39" s="12">
         <f>SUM(B35:B38)</f>
         <v/>
       </c>
-      <c r="C39" s="13">
+      <c r="C39" s="12">
         <f>SUM(C35:C38)</f>
         <v/>
       </c>
-      <c r="D39" s="13">
+      <c r="D39" s="12">
         <f>SUM(D35:D38)</f>
         <v/>
       </c>
@@ -1138,7 +1165,7 @@
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>3. FUNÇÃO OBJETIVO (Minimizar Custo Total)</t>
+          <t>3. FUNÇÃO OBJETIVO — Minimizar Custo Total</t>
         </is>
       </c>
       <c r="B41" s="3" t="n"/>
@@ -1152,10 +1179,10 @@
     <row r="43">
       <c r="A43" s="4" t="inlineStr">
         <is>
-          <t>Custo Fixo Total:</t>
-        </is>
-      </c>
-      <c r="B43" s="14">
+          <t>Custo Fixo:</t>
+        </is>
+      </c>
+      <c r="B43" s="13">
         <f>B14*A31+B15*B31+B16*C31+B17*D31</f>
         <v/>
       </c>
@@ -1163,21 +1190,21 @@
     <row r="44">
       <c r="A44" s="4" t="inlineStr">
         <is>
-          <t>Custo Variável Total:</t>
-        </is>
-      </c>
-      <c r="B44" s="14">
+          <t>Custo Variável:</t>
+        </is>
+      </c>
+      <c r="B44" s="13">
         <f>SUMPRODUCT(B7:D10,B35:D38)</f>
         <v/>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="15" t="inlineStr">
-        <is>
-          <t>CUSTO TOTAL (FO):</t>
-        </is>
-      </c>
-      <c r="B45" s="16">
+      <c r="A45" s="14" t="inlineStr">
+        <is>
+          <t>▶ CUSTO TOTAL (Célula Objetivo):</t>
+        </is>
+      </c>
+      <c r="B45" s="15">
         <f>B43+B44</f>
         <v/>
       </c>
@@ -1185,7 +1212,7 @@
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>4. RESTRIÇÕES</t>
+          <t>4. RESTRIÇÕES (LHS e RHS para o Solver)</t>
         </is>
       </c>
       <c r="B47" s="3" t="n"/>
@@ -1199,473 +1226,932 @@
     <row r="49">
       <c r="A49" s="5" t="inlineStr">
         <is>
-          <t>Restrição</t>
+          <t>Descrição</t>
         </is>
       </c>
       <c r="B49" s="5" t="inlineStr">
         <is>
-          <t>LHS</t>
+          <t>Célula LHS</t>
         </is>
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
+          <t>Fórmula LHS</t>
+        </is>
+      </c>
+      <c r="D49" s="5" t="inlineStr">
+        <is>
           <t>Sinal</t>
         </is>
       </c>
-      <c r="D49" s="5" t="inlineStr">
-        <is>
-          <t>RHS</t>
-        </is>
-      </c>
       <c r="E49" s="5" t="inlineStr">
         <is>
-          <t>Atendida?</t>
+          <t>Célula RHS</t>
+        </is>
+      </c>
+      <c r="F49" s="5" t="inlineStr">
+        <is>
+          <t>Valor RHS</t>
+        </is>
+      </c>
+      <c r="G49" s="5" t="inlineStr">
+        <is>
+          <t>Status</t>
         </is>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="17" t="inlineStr">
+      <c r="A50" s="16" t="inlineStr">
+        <is>
+          <t>Demanda Região 1: Σx_ij ≥ 8000</t>
+        </is>
+      </c>
+      <c r="B50" s="6" t="inlineStr">
+        <is>
+          <t>C50</t>
+        </is>
+      </c>
+      <c r="C50" s="12">
+        <f>B39</f>
+        <v/>
+      </c>
+      <c r="D50" s="17" t="inlineStr">
+        <is>
+          <t>&gt;=</t>
+        </is>
+      </c>
+      <c r="E50" s="6" t="inlineStr">
+        <is>
+          <t>F50</t>
+        </is>
+      </c>
+      <c r="F50" s="8" t="n">
+        <v>8000</v>
+      </c>
+      <c r="G50" s="18">
+        <f>IF(C50&gt;=F50,"OK","VIOLA")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="16" t="inlineStr">
+        <is>
+          <t>Demanda Região 2: Σx_ij ≥ 9000</t>
+        </is>
+      </c>
+      <c r="B51" s="6" t="inlineStr">
+        <is>
+          <t>C51</t>
+        </is>
+      </c>
+      <c r="C51" s="12">
+        <f>C39</f>
+        <v/>
+      </c>
+      <c r="D51" s="17" t="inlineStr">
+        <is>
+          <t>&gt;=</t>
+        </is>
+      </c>
+      <c r="E51" s="6" t="inlineStr">
+        <is>
+          <t>F51</t>
+        </is>
+      </c>
+      <c r="F51" s="8" t="n">
+        <v>9000</v>
+      </c>
+      <c r="G51" s="18">
+        <f>IF(C51&gt;=F51,"OK","VIOLA")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="16" t="inlineStr">
+        <is>
+          <t>Demanda Região 3: Σx_ij ≥ 7000</t>
+        </is>
+      </c>
+      <c r="B52" s="6" t="inlineStr">
+        <is>
+          <t>C52</t>
+        </is>
+      </c>
+      <c r="C52" s="12">
+        <f>D39</f>
+        <v/>
+      </c>
+      <c r="D52" s="17" t="inlineStr">
+        <is>
+          <t>&gt;=</t>
+        </is>
+      </c>
+      <c r="E52" s="6" t="inlineStr">
+        <is>
+          <t>F52</t>
+        </is>
+      </c>
+      <c r="F52" s="8" t="n">
+        <v>7000</v>
+      </c>
+      <c r="G52" s="18">
+        <f>IF(C52&gt;=F52,"OK","VIOLA")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="16" t="inlineStr">
+        <is>
+          <t>Capacidade NY: Σx_NYj ≤ 15000·y_NY</t>
+        </is>
+      </c>
+      <c r="B53" s="6" t="inlineStr">
+        <is>
+          <t>C53</t>
+        </is>
+      </c>
+      <c r="C53" s="12">
+        <f>E35</f>
+        <v/>
+      </c>
+      <c r="D53" s="17" t="inlineStr">
+        <is>
+          <t>&lt;=</t>
+        </is>
+      </c>
+      <c r="E53" s="6" t="inlineStr">
+        <is>
+          <t>F53</t>
+        </is>
+      </c>
+      <c r="F53" s="12">
+        <f>B25*A31</f>
+        <v/>
+      </c>
+      <c r="G53" s="18">
+        <f>IF(C53&lt;=F53,"OK","VIOLA")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="16" t="inlineStr">
+        <is>
+          <t>Capacidade LA: Σx_LAj ≤ 15000·y_LA</t>
+        </is>
+      </c>
+      <c r="B54" s="6" t="inlineStr">
+        <is>
+          <t>C54</t>
+        </is>
+      </c>
+      <c r="C54" s="12">
+        <f>E36</f>
+        <v/>
+      </c>
+      <c r="D54" s="17" t="inlineStr">
+        <is>
+          <t>&lt;=</t>
+        </is>
+      </c>
+      <c r="E54" s="6" t="inlineStr">
+        <is>
+          <t>F54</t>
+        </is>
+      </c>
+      <c r="F54" s="12">
+        <f>B25*B31</f>
+        <v/>
+      </c>
+      <c r="G54" s="18">
+        <f>IF(C54&lt;=F54,"OK","VIOLA")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="16" t="inlineStr">
+        <is>
+          <t>Capacidade Chicago: Σx_Chicagoj ≤ 15000·y_Chicago</t>
+        </is>
+      </c>
+      <c r="B55" s="6" t="inlineStr">
+        <is>
+          <t>C55</t>
+        </is>
+      </c>
+      <c r="C55" s="12">
+        <f>E37</f>
+        <v/>
+      </c>
+      <c r="D55" s="17" t="inlineStr">
+        <is>
+          <t>&lt;=</t>
+        </is>
+      </c>
+      <c r="E55" s="6" t="inlineStr">
+        <is>
+          <t>F55</t>
+        </is>
+      </c>
+      <c r="F55" s="12">
+        <f>B25*C31</f>
+        <v/>
+      </c>
+      <c r="G55" s="18">
+        <f>IF(C55&lt;=F55,"OK","VIOLA")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="16" t="inlineStr">
+        <is>
+          <t>Capacidade Atlanta: Σx_Atlantaj ≤ 15000·y_Atlanta</t>
+        </is>
+      </c>
+      <c r="B56" s="6" t="inlineStr">
+        <is>
+          <t>C56</t>
+        </is>
+      </c>
+      <c r="C56" s="12">
+        <f>E38</f>
+        <v/>
+      </c>
+      <c r="D56" s="17" t="inlineStr">
+        <is>
+          <t>&lt;=</t>
+        </is>
+      </c>
+      <c r="E56" s="6" t="inlineStr">
+        <is>
+          <t>F56</t>
+        </is>
+      </c>
+      <c r="F56" s="12">
+        <f>B25*D31</f>
+        <v/>
+      </c>
+      <c r="G56" s="18">
+        <f>IF(C56&lt;=F56,"OK","VIOLA")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="16" t="inlineStr">
+        <is>
+          <t>NY→LA: y_NY ≤ y_LA</t>
+        </is>
+      </c>
+      <c r="B57" s="6" t="inlineStr">
+        <is>
+          <t>C57</t>
+        </is>
+      </c>
+      <c r="C57" s="12">
+        <f>A31</f>
+        <v/>
+      </c>
+      <c r="D57" s="17" t="inlineStr">
+        <is>
+          <t>&lt;=</t>
+        </is>
+      </c>
+      <c r="E57" s="6" t="inlineStr">
+        <is>
+          <t>F57</t>
+        </is>
+      </c>
+      <c r="F57" s="12">
+        <f>B31</f>
+        <v/>
+      </c>
+      <c r="G57" s="18">
+        <f>IF(C57&lt;=F57,"OK","VIOLA")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="16" t="inlineStr">
+        <is>
+          <t>Máx 2 armazéns: Σy_i ≤ 2</t>
+        </is>
+      </c>
+      <c r="B58" s="6" t="inlineStr">
+        <is>
+          <t>C58</t>
+        </is>
+      </c>
+      <c r="C58" s="12">
+        <f>SUM(A31:D31)</f>
+        <v/>
+      </c>
+      <c r="D58" s="17" t="inlineStr">
+        <is>
+          <t>&lt;=</t>
+        </is>
+      </c>
+      <c r="E58" s="6" t="inlineStr">
+        <is>
+          <t>F58</t>
+        </is>
+      </c>
+      <c r="F58" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="G58" s="18">
+        <f>IF(C58&lt;=F58,"OK","VIOLA")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="16" t="inlineStr">
+        <is>
+          <t>ATL ou LA: y_ATL + y_LA ≥ 1</t>
+        </is>
+      </c>
+      <c r="B59" s="6" t="inlineStr">
+        <is>
+          <t>C59</t>
+        </is>
+      </c>
+      <c r="C59" s="12">
+        <f>D31+B31</f>
+        <v/>
+      </c>
+      <c r="D59" s="17" t="inlineStr">
+        <is>
+          <t>&gt;=</t>
+        </is>
+      </c>
+      <c r="E59" s="6" t="inlineStr">
+        <is>
+          <t>F59</t>
+        </is>
+      </c>
+      <c r="F59" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="G59" s="18">
+        <f>IF(C59&gt;=F59,"OK","VIOLA")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="19" t="inlineStr">
+        <is>
+          <t>y_i ∈ {0,1} — Binário</t>
+        </is>
+      </c>
+      <c r="B60" s="6" t="inlineStr">
+        <is>
+          <t>A31:D31</t>
+        </is>
+      </c>
+      <c r="D60" s="17" t="inlineStr">
+        <is>
+          <t>bin</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="19" t="inlineStr">
+        <is>
+          <t>x_ij ≥ 0 — Não-negatividade</t>
+        </is>
+      </c>
+      <c r="B61" s="6" t="inlineStr">
+        <is>
+          <t>B35:D38</t>
+        </is>
+      </c>
+      <c r="D61" s="17" t="inlineStr">
+        <is>
+          <t>&gt;=</t>
+        </is>
+      </c>
+      <c r="F61" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>5. CONFIGURAÇÃO DO SOLVER — PASSO A PASSO</t>
+        </is>
+      </c>
+      <c r="B63" s="3" t="n"/>
+      <c r="C63" s="3" t="n"/>
+      <c r="D63" s="3" t="n"/>
+      <c r="E63" s="3" t="n"/>
+      <c r="F63" s="3" t="n"/>
+      <c r="G63" s="3" t="n"/>
+      <c r="H63" s="3" t="n"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="20" t="inlineStr">
+        <is>
+          <t>PASSO 1:</t>
+        </is>
+      </c>
+      <c r="B65" s="21" t="inlineStr">
+        <is>
+          <t>Abra a aba 'Dados' → clique em 'Solver' (canto superior direito)</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="20" t="inlineStr">
+        <is>
+          <t>PASSO 2:</t>
+        </is>
+      </c>
+      <c r="B66" s="21" t="inlineStr">
+        <is>
+          <t>Definir Objetivo: selecione a célula B45 (custo total, fundo amarelo)</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="20" t="inlineStr">
+        <is>
+          <t>PASSO 3:</t>
+        </is>
+      </c>
+      <c r="B67" s="21" t="inlineStr">
+        <is>
+          <t>Para: selecione 'Mín' (minimizar)</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="20" t="inlineStr">
+        <is>
+          <t>PASSO 4:</t>
+        </is>
+      </c>
+      <c r="B68" s="21" t="inlineStr">
+        <is>
+          <t>Alterando Células Variáveis: A31:D31,B35:D38</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="20" t="inlineStr">
+        <is>
+          <t>PASSO 5:</t>
+        </is>
+      </c>
+      <c r="B69" s="21" t="inlineStr">
+        <is>
+          <t>Sujeito às Restrições — clique 'Adicionar' para cada uma:</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="4" t="inlineStr">
+        <is>
+          <t>Restrições a adicionar no Solver:</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="5" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B72" s="5" t="inlineStr">
+        <is>
+          <t>Referência da Célula (LHS)</t>
+        </is>
+      </c>
+      <c r="C72" s="5" t="inlineStr">
+        <is>
+          <t>Operador</t>
+        </is>
+      </c>
+      <c r="D72" s="5" t="inlineStr">
+        <is>
+          <t>Restrição (RHS)</t>
+        </is>
+      </c>
+      <c r="E72" s="5" t="inlineStr">
+        <is>
+          <t>Descrição</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="B73" s="22" t="inlineStr">
+        <is>
+          <t>C50</t>
+        </is>
+      </c>
+      <c r="C73" s="17" t="inlineStr">
+        <is>
+          <t>&gt;=</t>
+        </is>
+      </c>
+      <c r="D73" s="22" t="inlineStr">
+        <is>
+          <t>F50</t>
+        </is>
+      </c>
+      <c r="E73" s="16" t="inlineStr">
         <is>
           <t>Demanda Região 1</t>
         </is>
       </c>
-      <c r="B50" s="18">
-        <f>B39</f>
-        <v/>
-      </c>
-      <c r="C50" s="19" t="inlineStr">
+    </row>
+    <row r="74">
+      <c r="A74" s="18" t="n">
+        <v>2</v>
+      </c>
+      <c r="B74" s="22" t="inlineStr">
+        <is>
+          <t>C51</t>
+        </is>
+      </c>
+      <c r="C74" s="17" t="inlineStr">
         <is>
           <t>&gt;=</t>
         </is>
       </c>
-      <c r="D50" s="20" t="n">
-        <v>8000</v>
-      </c>
-      <c r="E50" s="19">
-        <f>IF(B50&gt;=D50,"OK","VIOLA")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="17" t="inlineStr">
+      <c r="D74" s="22" t="inlineStr">
+        <is>
+          <t>F51</t>
+        </is>
+      </c>
+      <c r="E74" s="16" t="inlineStr">
         <is>
           <t>Demanda Região 2</t>
         </is>
       </c>
-      <c r="B51" s="18">
-        <f>C39</f>
-        <v/>
-      </c>
-      <c r="C51" s="19" t="inlineStr">
+    </row>
+    <row r="75">
+      <c r="A75" s="18" t="n">
+        <v>3</v>
+      </c>
+      <c r="B75" s="22" t="inlineStr">
+        <is>
+          <t>C52</t>
+        </is>
+      </c>
+      <c r="C75" s="17" t="inlineStr">
         <is>
           <t>&gt;=</t>
         </is>
       </c>
-      <c r="D51" s="20" t="n">
-        <v>9000</v>
-      </c>
-      <c r="E51" s="19">
-        <f>IF(B51&gt;=D51,"OK","VIOLA")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="17" t="inlineStr">
+      <c r="D75" s="22" t="inlineStr">
+        <is>
+          <t>F52</t>
+        </is>
+      </c>
+      <c r="E75" s="16" t="inlineStr">
         <is>
           <t>Demanda Região 3</t>
         </is>
       </c>
-      <c r="B52" s="18">
-        <f>D39</f>
-        <v/>
-      </c>
-      <c r="C52" s="19" t="inlineStr">
+    </row>
+    <row r="76">
+      <c r="A76" s="18" t="n">
+        <v>4</v>
+      </c>
+      <c r="B76" s="22" t="inlineStr">
+        <is>
+          <t>C53</t>
+        </is>
+      </c>
+      <c r="C76" s="17" t="inlineStr">
+        <is>
+          <t>&lt;=</t>
+        </is>
+      </c>
+      <c r="D76" s="22" t="inlineStr">
+        <is>
+          <t>F53</t>
+        </is>
+      </c>
+      <c r="E76" s="16" t="inlineStr">
+        <is>
+          <t>Capacidade NY</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="18" t="n">
+        <v>5</v>
+      </c>
+      <c r="B77" s="22" t="inlineStr">
+        <is>
+          <t>C54</t>
+        </is>
+      </c>
+      <c r="C77" s="17" t="inlineStr">
+        <is>
+          <t>&lt;=</t>
+        </is>
+      </c>
+      <c r="D77" s="22" t="inlineStr">
+        <is>
+          <t>F54</t>
+        </is>
+      </c>
+      <c r="E77" s="16" t="inlineStr">
+        <is>
+          <t>Capacidade LA</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="18" t="n">
+        <v>6</v>
+      </c>
+      <c r="B78" s="22" t="inlineStr">
+        <is>
+          <t>C55</t>
+        </is>
+      </c>
+      <c r="C78" s="17" t="inlineStr">
+        <is>
+          <t>&lt;=</t>
+        </is>
+      </c>
+      <c r="D78" s="22" t="inlineStr">
+        <is>
+          <t>F55</t>
+        </is>
+      </c>
+      <c r="E78" s="16" t="inlineStr">
+        <is>
+          <t>Capacidade Chicago</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="18" t="n">
+        <v>7</v>
+      </c>
+      <c r="B79" s="22" t="inlineStr">
+        <is>
+          <t>C56</t>
+        </is>
+      </c>
+      <c r="C79" s="17" t="inlineStr">
+        <is>
+          <t>&lt;=</t>
+        </is>
+      </c>
+      <c r="D79" s="22" t="inlineStr">
+        <is>
+          <t>F56</t>
+        </is>
+      </c>
+      <c r="E79" s="16" t="inlineStr">
+        <is>
+          <t>Capacidade Atlanta</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="18" t="n">
+        <v>8</v>
+      </c>
+      <c r="B80" s="22" t="inlineStr">
+        <is>
+          <t>C57</t>
+        </is>
+      </c>
+      <c r="C80" s="17" t="inlineStr">
+        <is>
+          <t>&lt;=</t>
+        </is>
+      </c>
+      <c r="D80" s="22" t="inlineStr">
+        <is>
+          <t>F57</t>
+        </is>
+      </c>
+      <c r="E80" s="16" t="inlineStr">
+        <is>
+          <t>NY implica LA</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="18" t="n">
+        <v>9</v>
+      </c>
+      <c r="B81" s="22" t="inlineStr">
+        <is>
+          <t>C58</t>
+        </is>
+      </c>
+      <c r="C81" s="17" t="inlineStr">
+        <is>
+          <t>&lt;=</t>
+        </is>
+      </c>
+      <c r="D81" s="22" t="inlineStr">
+        <is>
+          <t>F58</t>
+        </is>
+      </c>
+      <c r="E81" s="16" t="inlineStr">
+        <is>
+          <t>Máx 2 armazéns</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="18" t="n">
+        <v>10</v>
+      </c>
+      <c r="B82" s="22" t="inlineStr">
+        <is>
+          <t>C59</t>
+        </is>
+      </c>
+      <c r="C82" s="17" t="inlineStr">
         <is>
           <t>&gt;=</t>
         </is>
       </c>
-      <c r="D52" s="20" t="n">
-        <v>7000</v>
-      </c>
-      <c r="E52" s="19">
-        <f>IF(B52&gt;=D52,"OK","VIOLA")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="17" t="inlineStr">
-        <is>
-          <t>Capacidade NY</t>
-        </is>
-      </c>
-      <c r="B53" s="18">
-        <f>E35</f>
-        <v/>
-      </c>
-      <c r="C53" s="19" t="inlineStr">
-        <is>
-          <t>&lt;=</t>
-        </is>
-      </c>
-      <c r="D53" s="18">
-        <f>B25*A31</f>
-        <v/>
-      </c>
-      <c r="E53" s="19">
-        <f>IF(B53&lt;=D53,"OK","VIOLA")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="17" t="inlineStr">
-        <is>
-          <t>Capacidade LA</t>
-        </is>
-      </c>
-      <c r="B54" s="18">
-        <f>E36</f>
-        <v/>
-      </c>
-      <c r="C54" s="19" t="inlineStr">
-        <is>
-          <t>&lt;=</t>
-        </is>
-      </c>
-      <c r="D54" s="18">
-        <f>B25*B31</f>
-        <v/>
-      </c>
-      <c r="E54" s="19">
-        <f>IF(B54&lt;=D54,"OK","VIOLA")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="17" t="inlineStr">
-        <is>
-          <t>Capacidade Chicago</t>
-        </is>
-      </c>
-      <c r="B55" s="18">
-        <f>E37</f>
-        <v/>
-      </c>
-      <c r="C55" s="19" t="inlineStr">
-        <is>
-          <t>&lt;=</t>
-        </is>
-      </c>
-      <c r="D55" s="18">
-        <f>B25*C31</f>
-        <v/>
-      </c>
-      <c r="E55" s="19">
-        <f>IF(B55&lt;=D55,"OK","VIOLA")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="17" t="inlineStr">
-        <is>
-          <t>Capacidade Atlanta</t>
-        </is>
-      </c>
-      <c r="B56" s="18">
-        <f>E38</f>
-        <v/>
-      </c>
-      <c r="C56" s="19" t="inlineStr">
-        <is>
-          <t>&lt;=</t>
-        </is>
-      </c>
-      <c r="D56" s="18">
-        <f>B25*D31</f>
-        <v/>
-      </c>
-      <c r="E56" s="19">
-        <f>IF(B56&lt;=D56,"OK","VIOLA")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="17" t="inlineStr">
-        <is>
-          <t>NY → LA (y_NY ≤ y_LA)</t>
-        </is>
-      </c>
-      <c r="B57" s="21">
-        <f>A31</f>
-        <v/>
-      </c>
-      <c r="C57" s="19" t="inlineStr">
-        <is>
-          <t>&lt;=</t>
-        </is>
-      </c>
-      <c r="D57" s="21">
-        <f>B31</f>
-        <v/>
-      </c>
-      <c r="E57" s="19">
-        <f>IF(B57&lt;=D57,"OK","VIOLA")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="17" t="inlineStr">
-        <is>
-          <t>Máx 2 armazéns (Σy ≤ 2)</t>
-        </is>
-      </c>
-      <c r="B58" s="21">
-        <f>SUM(A31:D31)</f>
-        <v/>
-      </c>
-      <c r="C58" s="19" t="inlineStr">
-        <is>
-          <t>&lt;=</t>
-        </is>
-      </c>
-      <c r="D58" s="22" t="n">
-        <v>2</v>
-      </c>
-      <c r="E58" s="19">
-        <f>IF(B58&lt;=D58,"OK","VIOLA")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="17" t="inlineStr">
-        <is>
-          <t>ATL ou LA (y_ATL + y_LA ≥ 1)</t>
-        </is>
-      </c>
-      <c r="B59" s="21">
-        <f>D31+B31</f>
-        <v/>
-      </c>
-      <c r="C59" s="19" t="inlineStr">
+      <c r="D82" s="22" t="inlineStr">
+        <is>
+          <t>F59</t>
+        </is>
+      </c>
+      <c r="E82" s="16" t="inlineStr">
+        <is>
+          <t>ATL ou LA</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="18" t="n">
+        <v>11</v>
+      </c>
+      <c r="B83" s="22" t="inlineStr">
+        <is>
+          <t>A31:D31</t>
+        </is>
+      </c>
+      <c r="C83" s="17" t="inlineStr">
+        <is>
+          <t>bin</t>
+        </is>
+      </c>
+      <c r="D83" s="22" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E83" s="16" t="inlineStr">
+        <is>
+          <t>Variáveis binárias</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="18" t="n">
+        <v>12</v>
+      </c>
+      <c r="B84" s="22" t="inlineStr">
+        <is>
+          <t>B35:D38</t>
+        </is>
+      </c>
+      <c r="C84" s="17" t="inlineStr">
         <is>
           <t>&gt;=</t>
         </is>
       </c>
-      <c r="D59" s="22" t="n">
-        <v>1</v>
-      </c>
-      <c r="E59" s="19">
-        <f>IF(B59&gt;=D59,"OK","VIOLA")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="17" t="inlineStr">
-        <is>
-          <t>y_i ∈ {0,1} (binário)</t>
-        </is>
-      </c>
-      <c r="B60" s="17" t="inlineStr">
-        <is>
-          <t>Restrição de tipo</t>
-        </is>
-      </c>
-      <c r="C60" s="19" t="inlineStr">
-        <is>
-          <t>=</t>
-        </is>
-      </c>
-      <c r="D60" s="23" t="inlineStr">
-        <is>
-          <t>Binário</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="2" t="inlineStr">
-        <is>
-          <t>5. CONFIGURAÇÃO DO SOLVER</t>
-        </is>
-      </c>
-      <c r="B62" s="3" t="n"/>
-      <c r="C62" s="3" t="n"/>
-      <c r="D62" s="3" t="n"/>
-      <c r="E62" s="3" t="n"/>
-      <c r="F62" s="3" t="n"/>
-      <c r="G62" s="3" t="n"/>
-      <c r="H62" s="3" t="n"/>
-    </row>
-    <row r="64">
-      <c r="A64" s="4" t="inlineStr">
-        <is>
-          <t>Célula Objetivo:</t>
-        </is>
-      </c>
-      <c r="B64" s="24" t="inlineStr">
-        <is>
-          <t>B45 (Minimizar)</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" s="4" t="inlineStr">
-        <is>
-          <t>Variáveis de Decisão:</t>
-        </is>
-      </c>
-      <c r="B65" s="24" t="inlineStr">
-        <is>
-          <t>A31:D31 (binárias), B35:D38 (contínuas)</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" s="4" t="inlineStr">
-        <is>
-          <t>Método:</t>
-        </is>
-      </c>
-      <c r="B66" s="24" t="inlineStr">
-        <is>
-          <t>Simplex LP (Branch &amp; Bound para variáveis binárias)</t>
-        </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" s="4" t="inlineStr">
-        <is>
-          <t>Restrições:</t>
-        </is>
-      </c>
-      <c r="B67" s="24" t="inlineStr"/>
-    </row>
-    <row r="68">
-      <c r="B68" s="24" t="inlineStr">
-        <is>
-          <t>B50 &gt;= D50  (Demanda Região 1)</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="B69" s="24" t="inlineStr">
-        <is>
-          <t>B51 &gt;= D51  (Demanda Região 2)</t>
-        </is>
-      </c>
-    </row>
-    <row r="70">
-      <c r="B70" s="24" t="inlineStr">
-        <is>
-          <t>B52 &gt;= D52  (Demanda Região 3)</t>
-        </is>
-      </c>
-    </row>
-    <row r="71">
-      <c r="B71" s="24" t="inlineStr">
-        <is>
-          <t>B53 &lt;= D53  (Capacidade NY)</t>
-        </is>
-      </c>
-    </row>
-    <row r="72">
-      <c r="B72" s="24" t="inlineStr">
-        <is>
-          <t>B54 &lt;= D54  (Capacidade LA)</t>
-        </is>
-      </c>
-    </row>
-    <row r="73">
-      <c r="B73" s="24" t="inlineStr">
-        <is>
-          <t>B55 &lt;= D55  (Capacidade Chicago)</t>
-        </is>
-      </c>
-    </row>
-    <row r="74">
-      <c r="B74" s="24" t="inlineStr">
-        <is>
-          <t>B56 &lt;= D56  (Capacidade Atlanta)</t>
-        </is>
-      </c>
-    </row>
-    <row r="75">
-      <c r="B75" s="24" t="inlineStr">
-        <is>
-          <t>B57 &lt;= D57  (NY→LA)</t>
-        </is>
-      </c>
-    </row>
-    <row r="76">
-      <c r="B76" s="24" t="inlineStr">
-        <is>
-          <t>B58 &lt;= D58  (Máx 2 armazéns)</t>
-        </is>
-      </c>
-    </row>
-    <row r="77">
-      <c r="B77" s="24" t="inlineStr">
-        <is>
-          <t>B59 &gt;= D59  (ATL ou LA)</t>
-        </is>
-      </c>
-    </row>
-    <row r="78">
-      <c r="B78" s="24" t="inlineStr">
-        <is>
-          <t>A31:D31 = Binário</t>
-        </is>
-      </c>
-    </row>
-    <row r="79">
-      <c r="B79" s="24" t="inlineStr">
-        <is>
-          <t>B35:D38 &gt;= 0</t>
-        </is>
-      </c>
-    </row>
-    <row r="82">
-      <c r="A82" s="2" t="inlineStr">
+      <c r="D84" s="22" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E84" s="16" t="inlineStr">
+        <is>
+          <t>Não-negatividade</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="20" t="inlineStr">
+        <is>
+          <t>PASSO 6:</t>
+        </is>
+      </c>
+      <c r="B86" s="4" t="inlineStr">
+        <is>
+          <t>Selecionar Método de Resolução: 'Simplex LP'</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="20" t="inlineStr">
+        <is>
+          <t>PASSO 7:</t>
+        </is>
+      </c>
+      <c r="B87" s="21" t="inlineStr">
+        <is>
+          <t>Marcar 'Tornar Variáveis Irrestritas Não Negativas' ✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="20" t="inlineStr">
+        <is>
+          <t>PASSO 8:</t>
+        </is>
+      </c>
+      <c r="B88" s="21" t="inlineStr">
+        <is>
+          <t>Clicar 'Resolver' → 'Manter Solução do Solver' → OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="23" t="inlineStr">
+        <is>
+          <t>NOTA:</t>
+        </is>
+      </c>
+      <c r="B90" s="24" t="inlineStr">
+        <is>
+          <t>O Excel usa Simplex LP com Branch &amp; Bound interno para variáveis binárias (inteiras). Não é necessário selecionar outro método — o Simplex LP do Solver trata binárias automaticamente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="91"/>
+    <row r="93">
+      <c r="A93" s="2" t="inlineStr">
         <is>
           <t>6. RESPOSTA POR EXTENSO</t>
         </is>
       </c>
-      <c r="B82" s="3" t="n"/>
-      <c r="C82" s="3" t="n"/>
-      <c r="D82" s="3" t="n"/>
-      <c r="E82" s="3" t="n"/>
-      <c r="F82" s="3" t="n"/>
-      <c r="G82" s="3" t="n"/>
-      <c r="H82" s="3" t="n"/>
-    </row>
-    <row r="84">
-      <c r="A84" s="25" t="inlineStr">
+      <c r="B93" s="3" t="n"/>
+      <c r="C93" s="3" t="n"/>
+      <c r="D93" s="3" t="n"/>
+      <c r="E93" s="3" t="n"/>
+      <c r="F93" s="3" t="n"/>
+      <c r="G93" s="3" t="n"/>
+      <c r="H93" s="3" t="n"/>
+    </row>
+    <row r="95">
+      <c r="A95" s="25" t="inlineStr">
         <is>
           <t>SOLUÇÃO ÓTIMA — Custo Total Mínimo: $751,000
 Armazéns abertos: LA, Chicago
-Envios (armazém → região):
-  LA → Região 2: 8,000 unidades
-  LA → Região 3: 7,000 unidades
-  Chicago → Região 1: 8,000 unidades
-  Chicago → Região 2: 1,000 unidades</t>
-        </is>
-      </c>
-    </row>
-    <row r="85"/>
-    <row r="86"/>
-    <row r="87"/>
-    <row r="88"/>
-    <row r="89"/>
-    <row r="90"/>
-    <row r="91"/>
-    <row r="92"/>
+Armazéns fechados: NY, Atlanta
+Distribuição ótima (armazém → região → quantidade):
+  • LA → Região 2: 8,000 unidades (custo unit.: $27)
+  • LA → Região 3: 7,000 unidades (custo unit.: $27)
+  • Chicago → Região 1: 8,000 unidades (custo unit.: $28)
+  • Chicago → Região 2: 1,000 unidades (custo unit.: $32)
+Verificação das restrições lógicas:
+  • NY aberto? Não, LA aberto? Sim → NY→LA: OK
+  • Total armazéns abertos: 2 ≤ 2 → OK
+  • ATL ou LA aberto? y_ATL+y_LA = 1 ≥ 1 → OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="96"/>
+    <row r="97"/>
+    <row r="98"/>
+    <row r="99"/>
+    <row r="100"/>
+    <row r="101"/>
+    <row r="102"/>
+    <row r="103"/>
+    <row r="104"/>
+    <row r="105"/>
+    <row r="106"/>
+    <row r="107"/>
+    <row r="108"/>
+    <row r="109"/>
   </sheetData>
-  <mergeCells count="9">
-    <mergeCell ref="A62:H62"/>
+  <mergeCells count="17">
+    <mergeCell ref="B66:H66"/>
     <mergeCell ref="A3:H3"/>
-    <mergeCell ref="A82:H82"/>
+    <mergeCell ref="B88:H88"/>
+    <mergeCell ref="B65:H65"/>
+    <mergeCell ref="B68:H68"/>
+    <mergeCell ref="A63:H63"/>
+    <mergeCell ref="B90:H91"/>
+    <mergeCell ref="B69:H69"/>
+    <mergeCell ref="B87:H87"/>
     <mergeCell ref="A41:H41"/>
+    <mergeCell ref="B86:H86"/>
+    <mergeCell ref="A95:H109"/>
     <mergeCell ref="A47:H47"/>
     <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A84:H92"/>
+    <mergeCell ref="A93:H93"/>
     <mergeCell ref="A27:H27"/>
     <mergeCell ref="B67:H67"/>
   </mergeCells>
@@ -1679,7 +2165,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K128"/>
+  <dimension ref="A1:K152"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1693,6 +2179,7 @@
     <col width="18" customWidth="1" min="9" max="9"/>
     <col width="18" customWidth="1" min="10" max="10"/>
     <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="18" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1722,7 +2209,7 @@
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>Arcos da Rede e Custos Padrão</t>
+          <t>Arcos da Rede — Custos Padrão e Ajustados por Tipo de Veículo</t>
         </is>
       </c>
     </row>
@@ -1744,7 +2231,7 @@
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>Custo Padrão</t>
+          <t>Custo Padrão ($)</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
@@ -1759,313 +2246,313 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="19" t="n">
+      <c r="A7" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="B7" s="23" t="inlineStr">
+      <c r="B7" s="26" t="inlineStr">
         <is>
           <t>Porto 1</t>
         </is>
       </c>
-      <c r="C7" s="23" t="inlineStr">
+      <c r="C7" s="26" t="inlineStr">
         <is>
           <t>Distrib. 1</t>
         </is>
       </c>
-      <c r="D7" s="26" t="n">
+      <c r="D7" s="27" t="n">
         <v>100</v>
       </c>
-      <c r="E7" s="27">
+      <c r="E7" s="28">
         <f>D7*1.15</f>
         <v/>
       </c>
-      <c r="F7" s="27">
+      <c r="F7" s="28">
         <f>D7*0.9</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="19" t="n">
+      <c r="A8" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="B8" s="23" t="inlineStr">
+      <c r="B8" s="26" t="inlineStr">
         <is>
           <t>Porto 1</t>
         </is>
       </c>
-      <c r="C8" s="23" t="inlineStr">
+      <c r="C8" s="26" t="inlineStr">
         <is>
           <t>Revenda 3</t>
         </is>
       </c>
-      <c r="D8" s="26" t="n">
+      <c r="D8" s="27" t="n">
         <v>300</v>
       </c>
-      <c r="E8" s="27">
+      <c r="E8" s="28">
         <f>D8*1.15</f>
         <v/>
       </c>
-      <c r="F8" s="27">
+      <c r="F8" s="28">
         <f>D8*0.9</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="19" t="n">
+      <c r="A9" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="B9" s="23" t="inlineStr">
+      <c r="B9" s="26" t="inlineStr">
         <is>
           <t>Porto 1</t>
         </is>
       </c>
-      <c r="C9" s="23" t="inlineStr">
+      <c r="C9" s="26" t="inlineStr">
         <is>
           <t>Distrib. 2</t>
         </is>
       </c>
-      <c r="D9" s="26" t="n">
+      <c r="D9" s="27" t="n">
         <v>130</v>
       </c>
-      <c r="E9" s="27">
+      <c r="E9" s="28">
         <f>D9*1.15</f>
         <v/>
       </c>
-      <c r="F9" s="27">
+      <c r="F9" s="28">
         <f>D9*0.9</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="19" t="n">
+      <c r="A10" s="18" t="n">
         <v>4</v>
       </c>
-      <c r="B10" s="23" t="inlineStr">
+      <c r="B10" s="26" t="inlineStr">
         <is>
           <t>Porto 2</t>
         </is>
       </c>
-      <c r="C10" s="23" t="inlineStr">
+      <c r="C10" s="26" t="inlineStr">
         <is>
           <t>Distrib. 1</t>
         </is>
       </c>
-      <c r="D10" s="26" t="n">
+      <c r="D10" s="27" t="n">
         <v>150</v>
       </c>
-      <c r="E10" s="27">
+      <c r="E10" s="28">
         <f>D10*1.15</f>
         <v/>
       </c>
-      <c r="F10" s="27">
+      <c r="F10" s="28">
         <f>D10*0.9</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="19" t="n">
+      <c r="A11" s="18" t="n">
         <v>5</v>
       </c>
-      <c r="B11" s="23" t="inlineStr">
+      <c r="B11" s="26" t="inlineStr">
         <is>
           <t>Porto 2</t>
         </is>
       </c>
-      <c r="C11" s="23" t="inlineStr">
+      <c r="C11" s="26" t="inlineStr">
         <is>
           <t>Revenda 2</t>
         </is>
       </c>
-      <c r="D11" s="26" t="n">
+      <c r="D11" s="27" t="n">
         <v>300</v>
       </c>
-      <c r="E11" s="27">
+      <c r="E11" s="28">
         <f>D11*1.15</f>
         <v/>
       </c>
-      <c r="F11" s="27">
+      <c r="F11" s="28">
         <f>D11*0.9</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="19" t="n">
+      <c r="A12" s="18" t="n">
         <v>6</v>
       </c>
-      <c r="B12" s="23" t="inlineStr">
+      <c r="B12" s="26" t="inlineStr">
         <is>
           <t>Porto 2</t>
         </is>
       </c>
-      <c r="C12" s="23" t="inlineStr">
+      <c r="C12" s="26" t="inlineStr">
         <is>
           <t>Distrib. 2</t>
         </is>
       </c>
-      <c r="D12" s="26" t="n">
+      <c r="D12" s="27" t="n">
         <v>120</v>
       </c>
-      <c r="E12" s="27">
+      <c r="E12" s="28">
         <f>D12*1.15</f>
         <v/>
       </c>
-      <c r="F12" s="27">
+      <c r="F12" s="28">
         <f>D12*0.9</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="19" t="n">
+      <c r="A13" s="18" t="n">
         <v>7</v>
       </c>
-      <c r="B13" s="23" t="inlineStr">
+      <c r="B13" s="26" t="inlineStr">
         <is>
           <t>Distrib. 1</t>
         </is>
       </c>
-      <c r="C13" s="23" t="inlineStr">
+      <c r="C13" s="26" t="inlineStr">
         <is>
           <t>Revenda 3</t>
         </is>
       </c>
-      <c r="D13" s="26" t="n">
+      <c r="D13" s="27" t="n">
         <v>160</v>
       </c>
-      <c r="E13" s="27">
+      <c r="E13" s="28">
         <f>D13*1.15</f>
         <v/>
       </c>
-      <c r="F13" s="27">
+      <c r="F13" s="28">
         <f>D13*0.9</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="19" t="n">
+      <c r="A14" s="18" t="n">
         <v>8</v>
       </c>
-      <c r="B14" s="23" t="inlineStr">
+      <c r="B14" s="26" t="inlineStr">
         <is>
           <t>Distrib. 1</t>
         </is>
       </c>
-      <c r="C14" s="23" t="inlineStr">
+      <c r="C14" s="26" t="inlineStr">
         <is>
           <t>Revenda 2</t>
         </is>
       </c>
-      <c r="D14" s="26" t="n">
+      <c r="D14" s="27" t="n">
         <v>170</v>
       </c>
-      <c r="E14" s="27">
+      <c r="E14" s="28">
         <f>D14*1.15</f>
         <v/>
       </c>
-      <c r="F14" s="27">
+      <c r="F14" s="28">
         <f>D14*0.9</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="19" t="n">
+      <c r="A15" s="18" t="n">
         <v>9</v>
       </c>
-      <c r="B15" s="23" t="inlineStr">
+      <c r="B15" s="26" t="inlineStr">
         <is>
           <t>Distrib. 1</t>
         </is>
       </c>
-      <c r="C15" s="23" t="inlineStr">
+      <c r="C15" s="26" t="inlineStr">
         <is>
           <t>Distrib. 2</t>
         </is>
       </c>
-      <c r="D15" s="26" t="n">
+      <c r="D15" s="27" t="n">
         <v>280</v>
       </c>
-      <c r="E15" s="27">
+      <c r="E15" s="28">
         <f>D15*1.15</f>
         <v/>
       </c>
-      <c r="F15" s="27">
+      <c r="F15" s="28">
         <f>D15*0.9</f>
         <v/>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="19" t="n">
+      <c r="A16" s="18" t="n">
         <v>10</v>
       </c>
-      <c r="B16" s="23" t="inlineStr">
+      <c r="B16" s="26" t="inlineStr">
         <is>
           <t>Distrib. 2</t>
         </is>
       </c>
-      <c r="C16" s="23" t="inlineStr">
+      <c r="C16" s="26" t="inlineStr">
         <is>
           <t>Revenda 3</t>
         </is>
       </c>
-      <c r="D16" s="26" t="n">
+      <c r="D16" s="27" t="n">
         <v>140</v>
       </c>
-      <c r="E16" s="27">
+      <c r="E16" s="28">
         <f>D16*1.15</f>
         <v/>
       </c>
-      <c r="F16" s="27">
+      <c r="F16" s="28">
         <f>D16*0.9</f>
         <v/>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="19" t="n">
+      <c r="A17" s="18" t="n">
         <v>11</v>
       </c>
-      <c r="B17" s="23" t="inlineStr">
+      <c r="B17" s="26" t="inlineStr">
         <is>
           <t>Distrib. 2</t>
         </is>
       </c>
-      <c r="C17" s="23" t="inlineStr">
+      <c r="C17" s="26" t="inlineStr">
         <is>
           <t>Revenda 2</t>
         </is>
       </c>
-      <c r="D17" s="26" t="n">
+      <c r="D17" s="27" t="n">
         <v>160</v>
       </c>
-      <c r="E17" s="27">
+      <c r="E17" s="28">
         <f>D17*1.15</f>
         <v/>
       </c>
-      <c r="F17" s="27">
+      <c r="F17" s="28">
         <f>D17*0.9</f>
         <v/>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="19" t="n">
+      <c r="A18" s="18" t="n">
         <v>12</v>
       </c>
-      <c r="B18" s="23" t="inlineStr">
+      <c r="B18" s="26" t="inlineStr">
         <is>
           <t>Revenda 3</t>
         </is>
       </c>
-      <c r="C18" s="23" t="inlineStr">
+      <c r="C18" s="26" t="inlineStr">
         <is>
           <t>Revenda 2</t>
         </is>
       </c>
-      <c r="D18" s="26" t="n">
+      <c r="D18" s="27" t="n">
         <v>150</v>
       </c>
-      <c r="E18" s="27">
+      <c r="E18" s="28">
         <f>D18*1.15</f>
         <v/>
       </c>
-      <c r="F18" s="27">
+      <c r="F18" s="28">
         <f>D18*0.9</f>
         <v/>
       </c>
@@ -2095,28 +2582,28 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="23" t="inlineStr">
+      <c r="A22" s="26" t="inlineStr">
         <is>
           <t>Porto 1</t>
         </is>
       </c>
-      <c r="B22" s="20" t="n">
+      <c r="B22" s="29" t="n">
         <v>325</v>
       </c>
-      <c r="C22" s="20" t="n">
+      <c r="C22" s="29" t="n">
         <v>450</v>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="23" t="inlineStr">
+      <c r="A23" s="26" t="inlineStr">
         <is>
           <t>Porto 2</t>
         </is>
       </c>
-      <c r="B23" s="20" t="n">
+      <c r="B23" s="29" t="n">
         <v>430</v>
       </c>
-      <c r="C23" s="20" t="n">
+      <c r="C23" s="29" t="n">
         <v>300</v>
       </c>
     </row>
@@ -2145,35 +2632,35 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="23" t="inlineStr">
+      <c r="A27" s="26" t="inlineStr">
         <is>
           <t>Revenda 3</t>
         </is>
       </c>
-      <c r="B27" s="20" t="n">
+      <c r="B27" s="29" t="n">
         <v>477</v>
       </c>
-      <c r="C27" s="20" t="n">
+      <c r="C27" s="29" t="n">
         <v>227</v>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="23" t="inlineStr">
+      <c r="A28" s="26" t="inlineStr">
         <is>
           <t>Revenda 2</t>
         </is>
       </c>
-      <c r="B28" s="20" t="n">
+      <c r="B28" s="29" t="n">
         <v>278</v>
       </c>
-      <c r="C28" s="20" t="n">
+      <c r="C28" s="29" t="n">
         <v>523</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>2. VARIÁVEIS DE DECISÃO (Fluxo por Arco e Tipo)</t>
+          <t>2. VARIÁVEIS DE DECISÃO — Fluxo por Arco (células que o Solver altera)</t>
         </is>
       </c>
       <c r="B31" s="3" t="n"/>
@@ -2190,7 +2677,7 @@
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
         <is>
-          <t>Fluxo de Veículos por Arco</t>
+          <t>Arco / Tipo de Veículo → Quantidades de Fluxo (variáveis) e Custos (fórmulas)</t>
         </is>
       </c>
     </row>
@@ -2227,460 +2714,460 @@
       </c>
       <c r="G34" s="5" t="inlineStr">
         <is>
-          <t>Custo Minivan</t>
+          <t>Custo Minivan ($)</t>
         </is>
       </c>
       <c r="H34" s="5" t="inlineStr">
         <is>
-          <t>Custo Esportivo</t>
+          <t>Custo Esportivo ($)</t>
         </is>
       </c>
       <c r="I34" s="5" t="inlineStr">
         <is>
-          <t>Custo Total Arco</t>
+          <t>Custo Total Arco ($)</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="19" t="n">
+      <c r="A35" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="B35" s="17" t="inlineStr">
+      <c r="B35" s="30" t="inlineStr">
         <is>
           <t>Porto 1</t>
         </is>
       </c>
-      <c r="C35" s="17" t="inlineStr">
+      <c r="C35" s="30" t="inlineStr">
         <is>
           <t>Distrib. 1</t>
         </is>
       </c>
-      <c r="D35" s="12" t="n">
+      <c r="D35" s="11" t="n">
         <v>325</v>
       </c>
-      <c r="E35" s="12" t="n">
+      <c r="E35" s="11" t="n">
         <v>450</v>
       </c>
-      <c r="F35" s="13">
+      <c r="F35" s="12">
         <f>D35+E35</f>
         <v/>
       </c>
-      <c r="G35" s="14">
+      <c r="G35" s="13">
         <f>D35*D7*1.15</f>
         <v/>
       </c>
-      <c r="H35" s="14">
+      <c r="H35" s="13">
         <f>E35*D7*0.9</f>
         <v/>
       </c>
-      <c r="I35" s="14">
+      <c r="I35" s="13">
         <f>G35+H35</f>
         <v/>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="19" t="n">
+      <c r="A36" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="B36" s="17" t="inlineStr">
+      <c r="B36" s="30" t="inlineStr">
         <is>
           <t>Porto 1</t>
         </is>
       </c>
-      <c r="C36" s="17" t="inlineStr">
+      <c r="C36" s="30" t="inlineStr">
         <is>
           <t>Revenda 3</t>
         </is>
       </c>
-      <c r="D36" s="12" t="n">
+      <c r="D36" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="E36" s="12" t="n">
+      <c r="E36" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="F36" s="13">
+      <c r="F36" s="12">
         <f>D36+E36</f>
         <v/>
       </c>
-      <c r="G36" s="14">
+      <c r="G36" s="13">
         <f>D36*D8*1.15</f>
         <v/>
       </c>
-      <c r="H36" s="14">
+      <c r="H36" s="13">
         <f>E36*D8*0.9</f>
         <v/>
       </c>
-      <c r="I36" s="14">
+      <c r="I36" s="13">
         <f>G36+H36</f>
         <v/>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="19" t="n">
+      <c r="A37" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="B37" s="17" t="inlineStr">
+      <c r="B37" s="30" t="inlineStr">
         <is>
           <t>Porto 1</t>
         </is>
       </c>
-      <c r="C37" s="17" t="inlineStr">
+      <c r="C37" s="30" t="inlineStr">
         <is>
           <t>Distrib. 2</t>
         </is>
       </c>
-      <c r="D37" s="12" t="n">
+      <c r="D37" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="E37" s="12" t="n">
+      <c r="E37" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="F37" s="13">
+      <c r="F37" s="12">
         <f>D37+E37</f>
         <v/>
       </c>
-      <c r="G37" s="14">
+      <c r="G37" s="13">
         <f>D37*D9*1.15</f>
         <v/>
       </c>
-      <c r="H37" s="14">
+      <c r="H37" s="13">
         <f>E37*D9*0.9</f>
         <v/>
       </c>
-      <c r="I37" s="14">
+      <c r="I37" s="13">
         <f>G37+H37</f>
         <v/>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="19" t="n">
+      <c r="A38" s="18" t="n">
         <v>4</v>
       </c>
-      <c r="B38" s="17" t="inlineStr">
+      <c r="B38" s="30" t="inlineStr">
         <is>
           <t>Porto 2</t>
         </is>
       </c>
-      <c r="C38" s="17" t="inlineStr">
+      <c r="C38" s="30" t="inlineStr">
         <is>
           <t>Distrib. 1</t>
         </is>
       </c>
-      <c r="D38" s="12" t="n">
+      <c r="D38" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="E38" s="12" t="n">
+      <c r="E38" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="F38" s="13">
+      <c r="F38" s="12">
         <f>D38+E38</f>
         <v/>
       </c>
-      <c r="G38" s="14">
+      <c r="G38" s="13">
         <f>D38*D10*1.15</f>
         <v/>
       </c>
-      <c r="H38" s="14">
+      <c r="H38" s="13">
         <f>E38*D10*0.9</f>
         <v/>
       </c>
-      <c r="I38" s="14">
+      <c r="I38" s="13">
         <f>G38+H38</f>
         <v/>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="19" t="n">
+      <c r="A39" s="18" t="n">
         <v>5</v>
       </c>
-      <c r="B39" s="17" t="inlineStr">
+      <c r="B39" s="30" t="inlineStr">
         <is>
           <t>Porto 2</t>
         </is>
       </c>
-      <c r="C39" s="17" t="inlineStr">
+      <c r="C39" s="30" t="inlineStr">
         <is>
           <t>Revenda 2</t>
         </is>
       </c>
-      <c r="D39" s="12" t="n">
+      <c r="D39" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="E39" s="12" t="n">
+      <c r="E39" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="F39" s="13">
+      <c r="F39" s="12">
         <f>D39+E39</f>
         <v/>
       </c>
-      <c r="G39" s="14">
+      <c r="G39" s="13">
         <f>D39*D11*1.15</f>
         <v/>
       </c>
-      <c r="H39" s="14">
+      <c r="H39" s="13">
         <f>E39*D11*0.9</f>
         <v/>
       </c>
-      <c r="I39" s="14">
+      <c r="I39" s="13">
         <f>G39+H39</f>
         <v/>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="19" t="n">
+      <c r="A40" s="18" t="n">
         <v>6</v>
       </c>
-      <c r="B40" s="17" t="inlineStr">
+      <c r="B40" s="30" t="inlineStr">
         <is>
           <t>Porto 2</t>
         </is>
       </c>
-      <c r="C40" s="17" t="inlineStr">
+      <c r="C40" s="30" t="inlineStr">
         <is>
           <t>Distrib. 2</t>
         </is>
       </c>
-      <c r="D40" s="12" t="n">
+      <c r="D40" s="11" t="n">
         <v>430</v>
       </c>
-      <c r="E40" s="12" t="n">
+      <c r="E40" s="11" t="n">
         <v>300</v>
       </c>
-      <c r="F40" s="13">
+      <c r="F40" s="12">
         <f>D40+E40</f>
         <v/>
       </c>
-      <c r="G40" s="14">
+      <c r="G40" s="13">
         <f>D40*D12*1.15</f>
         <v/>
       </c>
-      <c r="H40" s="14">
+      <c r="H40" s="13">
         <f>E40*D12*0.9</f>
         <v/>
       </c>
-      <c r="I40" s="14">
+      <c r="I40" s="13">
         <f>G40+H40</f>
         <v/>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="19" t="n">
+      <c r="A41" s="18" t="n">
         <v>7</v>
       </c>
-      <c r="B41" s="17" t="inlineStr">
+      <c r="B41" s="30" t="inlineStr">
         <is>
           <t>Distrib. 1</t>
         </is>
       </c>
-      <c r="C41" s="17" t="inlineStr">
+      <c r="C41" s="30" t="inlineStr">
         <is>
           <t>Revenda 3</t>
         </is>
       </c>
-      <c r="D41" s="12" t="n">
+      <c r="D41" s="11" t="n">
         <v>47</v>
       </c>
-      <c r="E41" s="12" t="n">
+      <c r="E41" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="F41" s="13">
+      <c r="F41" s="12">
         <f>D41+E41</f>
         <v/>
       </c>
-      <c r="G41" s="14">
+      <c r="G41" s="13">
         <f>D41*D13*1.15</f>
         <v/>
       </c>
-      <c r="H41" s="14">
+      <c r="H41" s="13">
         <f>E41*D13*0.9</f>
         <v/>
       </c>
-      <c r="I41" s="14">
+      <c r="I41" s="13">
         <f>G41+H41</f>
         <v/>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="19" t="n">
+      <c r="A42" s="18" t="n">
         <v>8</v>
       </c>
-      <c r="B42" s="17" t="inlineStr">
+      <c r="B42" s="30" t="inlineStr">
         <is>
           <t>Distrib. 1</t>
         </is>
       </c>
-      <c r="C42" s="17" t="inlineStr">
+      <c r="C42" s="30" t="inlineStr">
         <is>
           <t>Revenda 2</t>
         </is>
       </c>
-      <c r="D42" s="12" t="n">
+      <c r="D42" s="11" t="n">
         <v>278</v>
       </c>
-      <c r="E42" s="12" t="n">
+      <c r="E42" s="11" t="n">
         <v>450</v>
       </c>
-      <c r="F42" s="13">
+      <c r="F42" s="12">
         <f>D42+E42</f>
         <v/>
       </c>
-      <c r="G42" s="14">
+      <c r="G42" s="13">
         <f>D42*D14*1.15</f>
         <v/>
       </c>
-      <c r="H42" s="14">
+      <c r="H42" s="13">
         <f>E42*D14*0.9</f>
         <v/>
       </c>
-      <c r="I42" s="14">
+      <c r="I42" s="13">
         <f>G42+H42</f>
         <v/>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="19" t="n">
+      <c r="A43" s="18" t="n">
         <v>9</v>
       </c>
-      <c r="B43" s="17" t="inlineStr">
+      <c r="B43" s="30" t="inlineStr">
         <is>
           <t>Distrib. 1</t>
         </is>
       </c>
-      <c r="C43" s="17" t="inlineStr">
+      <c r="C43" s="30" t="inlineStr">
         <is>
           <t>Distrib. 2</t>
         </is>
       </c>
-      <c r="D43" s="12" t="n">
+      <c r="D43" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="E43" s="12" t="n">
+      <c r="E43" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="F43" s="13">
+      <c r="F43" s="12">
         <f>D43+E43</f>
         <v/>
       </c>
-      <c r="G43" s="14">
+      <c r="G43" s="13">
         <f>D43*D15*1.15</f>
         <v/>
       </c>
-      <c r="H43" s="14">
+      <c r="H43" s="13">
         <f>E43*D15*0.9</f>
         <v/>
       </c>
-      <c r="I43" s="14">
+      <c r="I43" s="13">
         <f>G43+H43</f>
         <v/>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="19" t="n">
+      <c r="A44" s="18" t="n">
         <v>10</v>
       </c>
-      <c r="B44" s="17" t="inlineStr">
+      <c r="B44" s="30" t="inlineStr">
         <is>
           <t>Distrib. 2</t>
         </is>
       </c>
-      <c r="C44" s="17" t="inlineStr">
+      <c r="C44" s="30" t="inlineStr">
         <is>
           <t>Revenda 3</t>
         </is>
       </c>
-      <c r="D44" s="12" t="n">
+      <c r="D44" s="11" t="n">
         <v>430</v>
       </c>
-      <c r="E44" s="12" t="n">
+      <c r="E44" s="11" t="n">
         <v>227</v>
       </c>
-      <c r="F44" s="13">
+      <c r="F44" s="12">
         <f>D44+E44</f>
         <v/>
       </c>
-      <c r="G44" s="14">
+      <c r="G44" s="13">
         <f>D44*D16*1.15</f>
         <v/>
       </c>
-      <c r="H44" s="14">
+      <c r="H44" s="13">
         <f>E44*D16*0.9</f>
         <v/>
       </c>
-      <c r="I44" s="14">
+      <c r="I44" s="13">
         <f>G44+H44</f>
         <v/>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="19" t="n">
+      <c r="A45" s="18" t="n">
         <v>11</v>
       </c>
-      <c r="B45" s="17" t="inlineStr">
+      <c r="B45" s="30" t="inlineStr">
         <is>
           <t>Distrib. 2</t>
         </is>
       </c>
-      <c r="C45" s="17" t="inlineStr">
+      <c r="C45" s="30" t="inlineStr">
         <is>
           <t>Revenda 2</t>
         </is>
       </c>
-      <c r="D45" s="12" t="n">
+      <c r="D45" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="E45" s="12" t="n">
+      <c r="E45" s="11" t="n">
         <v>73</v>
       </c>
-      <c r="F45" s="13">
+      <c r="F45" s="12">
         <f>D45+E45</f>
         <v/>
       </c>
-      <c r="G45" s="14">
+      <c r="G45" s="13">
         <f>D45*D17*1.15</f>
         <v/>
       </c>
-      <c r="H45" s="14">
+      <c r="H45" s="13">
         <f>E45*D17*0.9</f>
         <v/>
       </c>
-      <c r="I45" s="14">
+      <c r="I45" s="13">
         <f>G45+H45</f>
         <v/>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="19" t="n">
+      <c r="A46" s="18" t="n">
         <v>12</v>
       </c>
-      <c r="B46" s="17" t="inlineStr">
+      <c r="B46" s="30" t="inlineStr">
         <is>
           <t>Revenda 3</t>
         </is>
       </c>
-      <c r="C46" s="17" t="inlineStr">
+      <c r="C46" s="30" t="inlineStr">
         <is>
           <t>Revenda 2</t>
         </is>
       </c>
-      <c r="D46" s="12" t="n">
+      <c r="D46" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="E46" s="12" t="n">
+      <c r="E46" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="F46" s="13">
+      <c r="F46" s="12">
         <f>D46+E46</f>
         <v/>
       </c>
-      <c r="G46" s="14">
+      <c r="G46" s="13">
         <f>D46*D18*1.15</f>
         <v/>
       </c>
-      <c r="H46" s="14">
+      <c r="H46" s="13">
         <f>E46*D18*0.9</f>
         <v/>
       </c>
-      <c r="I46" s="14">
+      <c r="I46" s="13">
         <f>G46+H46</f>
         <v/>
       </c>
@@ -2688,7 +3175,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>3. FUNÇÃO OBJETIVO (Minimizar Custo Total de Transporte)</t>
+          <t>3. FUNÇÃO OBJETIVO — Minimizar Custo Total de Transporte</t>
         </is>
       </c>
       <c r="B48" s="3" t="n"/>
@@ -2703,12 +3190,12 @@
       <c r="K48" s="3" t="n"/>
     </row>
     <row r="50">
-      <c r="A50" s="15" t="inlineStr">
-        <is>
-          <t>CUSTO TOTAL (FO):</t>
-        </is>
-      </c>
-      <c r="B50" s="16">
+      <c r="A50" s="14" t="inlineStr">
+        <is>
+          <t>▶ CUSTO TOTAL (Célula Objetivo):</t>
+        </is>
+      </c>
+      <c r="B50" s="31">
         <f>SUM(I35:I46)</f>
         <v/>
       </c>
@@ -2716,7 +3203,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>4. RESTRIÇÕES</t>
+          <t>4. RESTRIÇÕES (LHS e RHS para o Solver)</t>
         </is>
       </c>
       <c r="B52" s="3" t="n"/>
@@ -2733,17 +3220,17 @@
     <row r="54">
       <c r="A54" s="5" t="inlineStr">
         <is>
-          <t>Restrição</t>
+          <t>Descrição</t>
         </is>
       </c>
       <c r="B54" s="5" t="inlineStr">
         <is>
-          <t>Tipo</t>
+          <t>Célula LHS</t>
         </is>
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
-          <t>LHS</t>
+          <t>Fórmula LHS</t>
         </is>
       </c>
       <c r="D54" s="5" t="inlineStr">
@@ -2753,708 +3240,1262 @@
       </c>
       <c r="E54" s="5" t="inlineStr">
         <is>
-          <t>RHS</t>
+          <t>Célula RHS</t>
         </is>
       </c>
       <c r="F54" s="5" t="inlineStr">
         <is>
-          <t>Atendida?</t>
+          <t>Valor RHS</t>
+        </is>
+      </c>
+      <c r="G54" s="5" t="inlineStr">
+        <is>
+          <t>Status</t>
         </is>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="17" t="inlineStr">
+      <c r="A55" s="16" t="inlineStr">
         <is>
           <t>Conservação Distrib. 1 (Minivan)</t>
         </is>
       </c>
-      <c r="B55" s="19" t="inlineStr">
-        <is>
-          <t>Fluxo</t>
-        </is>
-      </c>
-      <c r="C55" s="18">
+      <c r="B55" s="6" t="inlineStr">
+        <is>
+          <t>C55</t>
+        </is>
+      </c>
+      <c r="C55" s="12">
         <f>D35+D38-(D41+D42+D43)</f>
         <v/>
       </c>
-      <c r="D55" s="19" t="inlineStr">
+      <c r="D55" s="17" t="inlineStr">
         <is>
           <t>=</t>
         </is>
       </c>
-      <c r="E55" s="20" t="n">
+      <c r="E55" s="6" t="inlineStr">
+        <is>
+          <t>F55</t>
+        </is>
+      </c>
+      <c r="F55" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="F55" s="19">
-        <f>IF(C55=E55,"OK","VIOLA")</f>
+      <c r="G55" s="18">
+        <f>IF(ABS(C55-F55)&lt;0.01,"OK","VIOLA")</f>
         <v/>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="17" t="inlineStr">
+      <c r="A56" s="16" t="inlineStr">
         <is>
           <t>Conservação Distrib. 1 (Esportivo)</t>
         </is>
       </c>
-      <c r="B56" s="19" t="inlineStr">
-        <is>
-          <t>Fluxo</t>
-        </is>
-      </c>
-      <c r="C56" s="18">
+      <c r="B56" s="6" t="inlineStr">
+        <is>
+          <t>C56</t>
+        </is>
+      </c>
+      <c r="C56" s="12">
         <f>E35+E38-(E41+E42+E43)</f>
         <v/>
       </c>
-      <c r="D56" s="19" t="inlineStr">
+      <c r="D56" s="17" t="inlineStr">
         <is>
           <t>=</t>
         </is>
       </c>
-      <c r="E56" s="20" t="n">
+      <c r="E56" s="6" t="inlineStr">
+        <is>
+          <t>F56</t>
+        </is>
+      </c>
+      <c r="F56" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="F56" s="19">
-        <f>IF(C56=E56,"OK","VIOLA")</f>
+      <c r="G56" s="18">
+        <f>IF(ABS(C56-F56)&lt;0.01,"OK","VIOLA")</f>
         <v/>
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="17" t="inlineStr">
+      <c r="A57" s="16" t="inlineStr">
         <is>
           <t>Conservação Distrib. 2 (Minivan)</t>
         </is>
       </c>
-      <c r="B57" s="19" t="inlineStr">
-        <is>
-          <t>Fluxo</t>
-        </is>
-      </c>
-      <c r="C57" s="18">
+      <c r="B57" s="6" t="inlineStr">
+        <is>
+          <t>C57</t>
+        </is>
+      </c>
+      <c r="C57" s="12">
         <f>D37+D40+D43-(D44+D45)</f>
         <v/>
       </c>
-      <c r="D57" s="19" t="inlineStr">
+      <c r="D57" s="17" t="inlineStr">
         <is>
           <t>=</t>
         </is>
       </c>
-      <c r="E57" s="20" t="n">
+      <c r="E57" s="6" t="inlineStr">
+        <is>
+          <t>F57</t>
+        </is>
+      </c>
+      <c r="F57" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="F57" s="19">
-        <f>IF(C57=E57,"OK","VIOLA")</f>
+      <c r="G57" s="18">
+        <f>IF(ABS(C57-F57)&lt;0.01,"OK","VIOLA")</f>
         <v/>
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="17" t="inlineStr">
+      <c r="A58" s="16" t="inlineStr">
         <is>
           <t>Conservação Distrib. 2 (Esportivo)</t>
         </is>
       </c>
-      <c r="B58" s="19" t="inlineStr">
-        <is>
-          <t>Fluxo</t>
-        </is>
-      </c>
-      <c r="C58" s="18">
+      <c r="B58" s="6" t="inlineStr">
+        <is>
+          <t>C58</t>
+        </is>
+      </c>
+      <c r="C58" s="12">
         <f>E37+E40+E43-(E44+E45)</f>
         <v/>
       </c>
-      <c r="D58" s="19" t="inlineStr">
+      <c r="D58" s="17" t="inlineStr">
         <is>
           <t>=</t>
         </is>
       </c>
-      <c r="E58" s="20" t="n">
+      <c r="E58" s="6" t="inlineStr">
+        <is>
+          <t>F58</t>
+        </is>
+      </c>
+      <c r="F58" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="F58" s="19">
-        <f>IF(C58=E58,"OK","VIOLA")</f>
+      <c r="G58" s="18">
+        <f>IF(ABS(C58-F58)&lt;0.01,"OK","VIOLA")</f>
         <v/>
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="17" t="inlineStr">
+      <c r="A59" s="16" t="inlineStr">
         <is>
           <t>Oferta Porto 1 (Minivan)</t>
         </is>
       </c>
-      <c r="B59" s="19" t="inlineStr">
-        <is>
-          <t>Oferta</t>
-        </is>
-      </c>
-      <c r="C59" s="18">
+      <c r="B59" s="6" t="inlineStr">
+        <is>
+          <t>C59</t>
+        </is>
+      </c>
+      <c r="C59" s="12">
         <f>D35+D36+D37</f>
         <v/>
       </c>
-      <c r="D59" s="19" t="inlineStr">
+      <c r="D59" s="17" t="inlineStr">
         <is>
           <t>&lt;=</t>
         </is>
       </c>
-      <c r="E59" s="20" t="n">
+      <c r="E59" s="6" t="inlineStr">
+        <is>
+          <t>F59</t>
+        </is>
+      </c>
+      <c r="F59" s="8" t="n">
         <v>325</v>
       </c>
-      <c r="F59" s="19">
-        <f>IF(C59&lt;=E59,"OK","VIOLA")</f>
+      <c r="G59" s="18">
+        <f>IF(C59&lt;=F59,"OK","VIOLA")</f>
         <v/>
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="17" t="inlineStr">
+      <c r="A60" s="16" t="inlineStr">
         <is>
           <t>Oferta Porto 1 (Esportivo)</t>
         </is>
       </c>
-      <c r="B60" s="19" t="inlineStr">
-        <is>
-          <t>Oferta</t>
-        </is>
-      </c>
-      <c r="C60" s="18">
+      <c r="B60" s="6" t="inlineStr">
+        <is>
+          <t>C60</t>
+        </is>
+      </c>
+      <c r="C60" s="12">
         <f>E35+E36+E37</f>
         <v/>
       </c>
-      <c r="D60" s="19" t="inlineStr">
+      <c r="D60" s="17" t="inlineStr">
         <is>
           <t>&lt;=</t>
         </is>
       </c>
-      <c r="E60" s="20" t="n">
+      <c r="E60" s="6" t="inlineStr">
+        <is>
+          <t>F60</t>
+        </is>
+      </c>
+      <c r="F60" s="8" t="n">
         <v>450</v>
       </c>
-      <c r="F60" s="19">
-        <f>IF(C60&lt;=E60,"OK","VIOLA")</f>
+      <c r="G60" s="18">
+        <f>IF(C60&lt;=F60,"OK","VIOLA")</f>
         <v/>
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="17" t="inlineStr">
+      <c r="A61" s="16" t="inlineStr">
         <is>
           <t>Oferta Porto 2 (Minivan)</t>
         </is>
       </c>
-      <c r="B61" s="19" t="inlineStr">
-        <is>
-          <t>Oferta</t>
-        </is>
-      </c>
-      <c r="C61" s="18">
+      <c r="B61" s="6" t="inlineStr">
+        <is>
+          <t>C61</t>
+        </is>
+      </c>
+      <c r="C61" s="12">
         <f>D38+D39+D40</f>
         <v/>
       </c>
-      <c r="D61" s="19" t="inlineStr">
+      <c r="D61" s="17" t="inlineStr">
         <is>
           <t>&lt;=</t>
         </is>
       </c>
-      <c r="E61" s="20" t="n">
+      <c r="E61" s="6" t="inlineStr">
+        <is>
+          <t>F61</t>
+        </is>
+      </c>
+      <c r="F61" s="8" t="n">
         <v>430</v>
       </c>
-      <c r="F61" s="19">
-        <f>IF(C61&lt;=E61,"OK","VIOLA")</f>
+      <c r="G61" s="18">
+        <f>IF(C61&lt;=F61,"OK","VIOLA")</f>
         <v/>
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="17" t="inlineStr">
+      <c r="A62" s="16" t="inlineStr">
         <is>
           <t>Oferta Porto 2 (Esportivo)</t>
         </is>
       </c>
-      <c r="B62" s="19" t="inlineStr">
-        <is>
-          <t>Oferta</t>
-        </is>
-      </c>
-      <c r="C62" s="18">
+      <c r="B62" s="6" t="inlineStr">
+        <is>
+          <t>C62</t>
+        </is>
+      </c>
+      <c r="C62" s="12">
         <f>E38+E39+E40</f>
         <v/>
       </c>
-      <c r="D62" s="19" t="inlineStr">
+      <c r="D62" s="17" t="inlineStr">
         <is>
           <t>&lt;=</t>
         </is>
       </c>
-      <c r="E62" s="20" t="n">
+      <c r="E62" s="6" t="inlineStr">
+        <is>
+          <t>F62</t>
+        </is>
+      </c>
+      <c r="F62" s="8" t="n">
         <v>300</v>
       </c>
-      <c r="F62" s="19">
-        <f>IF(C62&lt;=E62,"OK","VIOLA")</f>
+      <c r="G62" s="18">
+        <f>IF(C62&lt;=F62,"OK","VIOLA")</f>
         <v/>
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="17" t="inlineStr">
+      <c r="A63" s="16" t="inlineStr">
         <is>
           <t>Demanda Revenda 3 (Minivan)</t>
         </is>
       </c>
-      <c r="B63" s="19" t="inlineStr">
-        <is>
-          <t>Demanda</t>
-        </is>
-      </c>
-      <c r="C63" s="18">
+      <c r="B63" s="6" t="inlineStr">
+        <is>
+          <t>C63</t>
+        </is>
+      </c>
+      <c r="C63" s="12">
         <f>D36+D41+D44-(D46)</f>
         <v/>
       </c>
-      <c r="D63" s="19" t="inlineStr">
+      <c r="D63" s="17" t="inlineStr">
         <is>
           <t>&gt;=</t>
         </is>
       </c>
-      <c r="E63" s="20" t="n">
+      <c r="E63" s="6" t="inlineStr">
+        <is>
+          <t>F63</t>
+        </is>
+      </c>
+      <c r="F63" s="8" t="n">
         <v>477</v>
       </c>
-      <c r="F63" s="19">
-        <f>IF(C63&gt;=E63,"OK","VIOLA")</f>
+      <c r="G63" s="18">
+        <f>IF(C63&gt;=F63,"OK","VIOLA")</f>
         <v/>
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="17" t="inlineStr">
+      <c r="A64" s="16" t="inlineStr">
         <is>
           <t>Demanda Revenda 3 (Esportivo)</t>
         </is>
       </c>
-      <c r="B64" s="19" t="inlineStr">
-        <is>
-          <t>Demanda</t>
-        </is>
-      </c>
-      <c r="C64" s="18">
+      <c r="B64" s="6" t="inlineStr">
+        <is>
+          <t>C64</t>
+        </is>
+      </c>
+      <c r="C64" s="12">
         <f>E36+E41+E44-(E46)</f>
         <v/>
       </c>
-      <c r="D64" s="19" t="inlineStr">
+      <c r="D64" s="17" t="inlineStr">
         <is>
           <t>&gt;=</t>
         </is>
       </c>
-      <c r="E64" s="20" t="n">
+      <c r="E64" s="6" t="inlineStr">
+        <is>
+          <t>F64</t>
+        </is>
+      </c>
+      <c r="F64" s="8" t="n">
         <v>227</v>
       </c>
-      <c r="F64" s="19">
-        <f>IF(C64&gt;=E64,"OK","VIOLA")</f>
+      <c r="G64" s="18">
+        <f>IF(C64&gt;=F64,"OK","VIOLA")</f>
         <v/>
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="17" t="inlineStr">
+      <c r="A65" s="16" t="inlineStr">
         <is>
           <t>Demanda Revenda 2 (Minivan)</t>
         </is>
       </c>
-      <c r="B65" s="19" t="inlineStr">
-        <is>
-          <t>Demanda</t>
-        </is>
-      </c>
-      <c r="C65" s="18">
+      <c r="B65" s="6" t="inlineStr">
+        <is>
+          <t>C65</t>
+        </is>
+      </c>
+      <c r="C65" s="12">
         <f>D39+D42+D45+D46-(0)</f>
         <v/>
       </c>
-      <c r="D65" s="19" t="inlineStr">
+      <c r="D65" s="17" t="inlineStr">
         <is>
           <t>&gt;=</t>
         </is>
       </c>
-      <c r="E65" s="20" t="n">
+      <c r="E65" s="6" t="inlineStr">
+        <is>
+          <t>F65</t>
+        </is>
+      </c>
+      <c r="F65" s="8" t="n">
         <v>278</v>
       </c>
-      <c r="F65" s="19">
-        <f>IF(C65&gt;=E65,"OK","VIOLA")</f>
+      <c r="G65" s="18">
+        <f>IF(C65&gt;=F65,"OK","VIOLA")</f>
         <v/>
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="17" t="inlineStr">
+      <c r="A66" s="16" t="inlineStr">
         <is>
           <t>Demanda Revenda 2 (Esportivo)</t>
         </is>
       </c>
-      <c r="B66" s="19" t="inlineStr">
-        <is>
-          <t>Demanda</t>
-        </is>
-      </c>
-      <c r="C66" s="18">
+      <c r="B66" s="6" t="inlineStr">
+        <is>
+          <t>C66</t>
+        </is>
+      </c>
+      <c r="C66" s="12">
         <f>E39+E42+E45+E46-(0)</f>
         <v/>
       </c>
-      <c r="D66" s="19" t="inlineStr">
+      <c r="D66" s="17" t="inlineStr">
         <is>
           <t>&gt;=</t>
         </is>
       </c>
-      <c r="E66" s="20" t="n">
+      <c r="E66" s="6" t="inlineStr">
+        <is>
+          <t>F66</t>
+        </is>
+      </c>
+      <c r="F66" s="8" t="n">
         <v>523</v>
       </c>
-      <c r="F66" s="19">
-        <f>IF(C66&gt;=E66,"OK","VIOLA")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" s="2" t="inlineStr">
-        <is>
-          <t>5. CONFIGURAÇÃO DO SOLVER</t>
-        </is>
-      </c>
-      <c r="B68" s="3" t="n"/>
-      <c r="C68" s="3" t="n"/>
-      <c r="D68" s="3" t="n"/>
-      <c r="E68" s="3" t="n"/>
-      <c r="F68" s="3" t="n"/>
-      <c r="G68" s="3" t="n"/>
-      <c r="H68" s="3" t="n"/>
-      <c r="I68" s="3" t="n"/>
-      <c r="J68" s="3" t="n"/>
-      <c r="K68" s="3" t="n"/>
-    </row>
-    <row r="70">
-      <c r="A70" s="4" t="inlineStr">
-        <is>
-          <t>Célula Objetivo:</t>
-        </is>
-      </c>
-      <c r="B70" s="24" t="inlineStr">
-        <is>
-          <t>B50 (Minimizar)</t>
-        </is>
-      </c>
+      <c r="G66" s="18">
+        <f>IF(C66&gt;=F66,"OK","VIOLA")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="19" t="inlineStr">
+        <is>
+          <t>f_ij_v ≥ 0 — Não-negatividade (todas variáveis)</t>
+        </is>
+      </c>
+      <c r="B67" s="6" t="inlineStr">
+        <is>
+          <t>D35:E46</t>
+        </is>
+      </c>
+      <c r="D67" s="17" t="inlineStr">
+        <is>
+          <t>&gt;=</t>
+        </is>
+      </c>
+      <c r="F67" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="inlineStr">
+        <is>
+          <t>5. CONFIGURAÇÃO DO SOLVER — PASSO A PASSO</t>
+        </is>
+      </c>
+      <c r="B69" s="3" t="n"/>
+      <c r="C69" s="3" t="n"/>
+      <c r="D69" s="3" t="n"/>
+      <c r="E69" s="3" t="n"/>
+      <c r="F69" s="3" t="n"/>
+      <c r="G69" s="3" t="n"/>
+      <c r="H69" s="3" t="n"/>
+      <c r="I69" s="3" t="n"/>
+      <c r="J69" s="3" t="n"/>
+      <c r="K69" s="3" t="n"/>
     </row>
     <row r="71">
-      <c r="A71" s="4" t="inlineStr">
-        <is>
-          <t>Variáveis de Decisão:</t>
+      <c r="A71" s="20" t="inlineStr">
+        <is>
+          <t>PASSO 1:</t>
         </is>
       </c>
       <c r="B71" s="24" t="inlineStr">
         <is>
-          <t>D35:E46 (fluxos contínuos ≥ 0)</t>
+          <t>Abra a aba 'Dados' → clique em 'Solver' (canto superior direito)</t>
         </is>
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="4" t="inlineStr">
-        <is>
-          <t>Método:</t>
+      <c r="A72" s="20" t="inlineStr">
+        <is>
+          <t>PASSO 2:</t>
         </is>
       </c>
       <c r="B72" s="24" t="inlineStr">
         <is>
-          <t>Simplex LP</t>
+          <t>Definir Objetivo: selecione a célula B50 (custo total, fundo amarelo)</t>
         </is>
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="4" t="inlineStr">
-        <is>
-          <t>Restrições:</t>
+      <c r="A73" s="20" t="inlineStr">
+        <is>
+          <t>PASSO 3:</t>
         </is>
       </c>
       <c r="B73" s="24" t="inlineStr">
         <is>
-          <t>Ver seção 4 acima — conservação de fluxo, oferta e demanda</t>
-        </is>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" s="2" t="inlineStr">
-        <is>
-          <t>6. RESPOSTAS POR EXTENSO (Itens c e d)</t>
-        </is>
-      </c>
-      <c r="B76" s="3" t="n"/>
-      <c r="C76" s="3" t="n"/>
-      <c r="D76" s="3" t="n"/>
-      <c r="E76" s="3" t="n"/>
-      <c r="F76" s="3" t="n"/>
-      <c r="G76" s="3" t="n"/>
-      <c r="H76" s="3" t="n"/>
-      <c r="I76" s="3" t="n"/>
-      <c r="J76" s="3" t="n"/>
-      <c r="K76" s="3" t="n"/>
+          <t>Para: selecione 'Mín' (minimizar)</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="20" t="inlineStr">
+        <is>
+          <t>PASSO 4:</t>
+        </is>
+      </c>
+      <c r="B74" s="24" t="inlineStr">
+        <is>
+          <t>Alterando Células Variáveis: D35:E35,D36:E36,...,D46:E46
+  → Ou simplesmente: D35:E46</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="20" t="inlineStr">
+        <is>
+          <t>PASSO 5:</t>
+        </is>
+      </c>
+      <c r="B75" s="24" t="inlineStr">
+        <is>
+          <t>Sujeito às Restrições — clique 'Adicionar' para cada uma (ver tabela abaixo):</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="4" t="inlineStr">
+        <is>
+          <t>Restrições a adicionar no Solver:</t>
+        </is>
+      </c>
     </row>
     <row r="78">
-      <c r="A78" s="25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ITEM c) Fluxo ótimo por tipo de veículo:
---- Minivan ---
-  Porto 1 → Distrib. 1: 325 veículos (custo unitário: $115.00)
-  Porto 2 → Distrib. 2: 430 veículos (custo unitário: $138.00)
-  Distrib. 1 → Revenda 3: 47 veículos (custo unitário: $184.00)
-  Distrib. 1 → Revenda 2: 278 veículos (custo unitário: $195.50)
-  Distrib. 2 → Revenda 3: 430 veículos (custo unitário: $161.00)
---- Esportivo ---
-  Porto 1 → Distrib. 1: 450 veículos (custo unitário: $90.00)
-  Porto 2 → Distrib. 2: 300 veículos (custo unitário: $108.00)
-  Distrib. 1 → Revenda 2: 450 veículos (custo unitário: $153.00)
-  Distrib. 2 → Revenda 3: 227 veículos (custo unitário: $126.00)
-  Distrib. 2 → Revenda 2: 73 veículos (custo unitário: $144.00)
+      <c r="A78" s="5" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B78" s="5" t="inlineStr">
+        <is>
+          <t>Referência da Célula (LHS)</t>
+        </is>
+      </c>
+      <c r="C78" s="5" t="inlineStr">
+        <is>
+          <t>Operador</t>
+        </is>
+      </c>
+      <c r="D78" s="5" t="inlineStr">
+        <is>
+          <t>Restrição (RHS)</t>
+        </is>
+      </c>
+      <c r="E78" s="5" t="inlineStr">
+        <is>
+          <t>Descrição</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="B79" s="22" t="inlineStr">
+        <is>
+          <t>C55</t>
+        </is>
+      </c>
+      <c r="C79" s="17" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="D79" s="22" t="inlineStr">
+        <is>
+          <t>F55</t>
+        </is>
+      </c>
+      <c r="E79" s="16" t="inlineStr">
+        <is>
+          <t>Conservação Distrib. 1 (Minivan)</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="18" t="n">
+        <v>2</v>
+      </c>
+      <c r="B80" s="22" t="inlineStr">
+        <is>
+          <t>C56</t>
+        </is>
+      </c>
+      <c r="C80" s="17" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="D80" s="22" t="inlineStr">
+        <is>
+          <t>F56</t>
+        </is>
+      </c>
+      <c r="E80" s="16" t="inlineStr">
+        <is>
+          <t>Conservação Distrib. 1 (Esportivo)</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="18" t="n">
+        <v>3</v>
+      </c>
+      <c r="B81" s="22" t="inlineStr">
+        <is>
+          <t>C57</t>
+        </is>
+      </c>
+      <c r="C81" s="17" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="D81" s="22" t="inlineStr">
+        <is>
+          <t>F57</t>
+        </is>
+      </c>
+      <c r="E81" s="16" t="inlineStr">
+        <is>
+          <t>Conservação Distrib. 2 (Minivan)</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="18" t="n">
+        <v>4</v>
+      </c>
+      <c r="B82" s="22" t="inlineStr">
+        <is>
+          <t>C58</t>
+        </is>
+      </c>
+      <c r="C82" s="17" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="D82" s="22" t="inlineStr">
+        <is>
+          <t>F58</t>
+        </is>
+      </c>
+      <c r="E82" s="16" t="inlineStr">
+        <is>
+          <t>Conservação Distrib. 2 (Esportivo)</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="18" t="n">
+        <v>5</v>
+      </c>
+      <c r="B83" s="22" t="inlineStr">
+        <is>
+          <t>C59</t>
+        </is>
+      </c>
+      <c r="C83" s="17" t="inlineStr">
+        <is>
+          <t>&lt;=</t>
+        </is>
+      </c>
+      <c r="D83" s="22" t="inlineStr">
+        <is>
+          <t>F59</t>
+        </is>
+      </c>
+      <c r="E83" s="16" t="inlineStr">
+        <is>
+          <t>Oferta Porto 1 (Minivan)</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="18" t="n">
+        <v>6</v>
+      </c>
+      <c r="B84" s="22" t="inlineStr">
+        <is>
+          <t>C60</t>
+        </is>
+      </c>
+      <c r="C84" s="17" t="inlineStr">
+        <is>
+          <t>&lt;=</t>
+        </is>
+      </c>
+      <c r="D84" s="22" t="inlineStr">
+        <is>
+          <t>F60</t>
+        </is>
+      </c>
+      <c r="E84" s="16" t="inlineStr">
+        <is>
+          <t>Oferta Porto 1 (Esportivo)</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="18" t="n">
+        <v>7</v>
+      </c>
+      <c r="B85" s="22" t="inlineStr">
+        <is>
+          <t>C61</t>
+        </is>
+      </c>
+      <c r="C85" s="17" t="inlineStr">
+        <is>
+          <t>&lt;=</t>
+        </is>
+      </c>
+      <c r="D85" s="22" t="inlineStr">
+        <is>
+          <t>F61</t>
+        </is>
+      </c>
+      <c r="E85" s="16" t="inlineStr">
+        <is>
+          <t>Oferta Porto 2 (Minivan)</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="18" t="n">
+        <v>8</v>
+      </c>
+      <c r="B86" s="22" t="inlineStr">
+        <is>
+          <t>C62</t>
+        </is>
+      </c>
+      <c r="C86" s="17" t="inlineStr">
+        <is>
+          <t>&lt;=</t>
+        </is>
+      </c>
+      <c r="D86" s="22" t="inlineStr">
+        <is>
+          <t>F62</t>
+        </is>
+      </c>
+      <c r="E86" s="16" t="inlineStr">
+        <is>
+          <t>Oferta Porto 2 (Esportivo)</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="18" t="n">
+        <v>9</v>
+      </c>
+      <c r="B87" s="22" t="inlineStr">
+        <is>
+          <t>C63</t>
+        </is>
+      </c>
+      <c r="C87" s="17" t="inlineStr">
+        <is>
+          <t>&gt;=</t>
+        </is>
+      </c>
+      <c r="D87" s="22" t="inlineStr">
+        <is>
+          <t>F63</t>
+        </is>
+      </c>
+      <c r="E87" s="16" t="inlineStr">
+        <is>
+          <t>Demanda Revenda 3 (Minivan)</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="18" t="n">
+        <v>10</v>
+      </c>
+      <c r="B88" s="22" t="inlineStr">
+        <is>
+          <t>C64</t>
+        </is>
+      </c>
+      <c r="C88" s="17" t="inlineStr">
+        <is>
+          <t>&gt;=</t>
+        </is>
+      </c>
+      <c r="D88" s="22" t="inlineStr">
+        <is>
+          <t>F64</t>
+        </is>
+      </c>
+      <c r="E88" s="16" t="inlineStr">
+        <is>
+          <t>Demanda Revenda 3 (Esportivo)</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="18" t="n">
+        <v>11</v>
+      </c>
+      <c r="B89" s="22" t="inlineStr">
+        <is>
+          <t>C65</t>
+        </is>
+      </c>
+      <c r="C89" s="17" t="inlineStr">
+        <is>
+          <t>&gt;=</t>
+        </is>
+      </c>
+      <c r="D89" s="22" t="inlineStr">
+        <is>
+          <t>F65</t>
+        </is>
+      </c>
+      <c r="E89" s="16" t="inlineStr">
+        <is>
+          <t>Demanda Revenda 2 (Minivan)</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="18" t="n">
+        <v>12</v>
+      </c>
+      <c r="B90" s="22" t="inlineStr">
+        <is>
+          <t>C66</t>
+        </is>
+      </c>
+      <c r="C90" s="17" t="inlineStr">
+        <is>
+          <t>&gt;=</t>
+        </is>
+      </c>
+      <c r="D90" s="22" t="inlineStr">
+        <is>
+          <t>F66</t>
+        </is>
+      </c>
+      <c r="E90" s="16" t="inlineStr">
+        <is>
+          <t>Demanda Revenda 2 (Esportivo)</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="18" t="n">
+        <v>13</v>
+      </c>
+      <c r="B91" s="22" t="inlineStr">
+        <is>
+          <t>D35:E46</t>
+        </is>
+      </c>
+      <c r="C91" s="17" t="inlineStr">
+        <is>
+          <t>&gt;=</t>
+        </is>
+      </c>
+      <c r="D91" s="22" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E91" s="16" t="inlineStr">
+        <is>
+          <t>Não-negatividade</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="20" t="inlineStr">
+        <is>
+          <t>PASSO 6:</t>
+        </is>
+      </c>
+      <c r="B93" s="4" t="inlineStr">
+        <is>
+          <t>Selecionar Método de Resolução: 'Simplex LP'</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="20" t="inlineStr">
+        <is>
+          <t>PASSO 7:</t>
+        </is>
+      </c>
+      <c r="B94" s="21" t="inlineStr">
+        <is>
+          <t>Marcar 'Tornar Variáveis Irrestritas Não Negativas' ✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="20" t="inlineStr">
+        <is>
+          <t>PASSO 8:</t>
+        </is>
+      </c>
+      <c r="B95" s="21" t="inlineStr">
+        <is>
+          <t>Clicar 'Resolver' → 'Manter Solução do Solver' → OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="inlineStr">
+        <is>
+          <t>6. RESPOSTAS POR EXTENSO — Itens c) e d)</t>
+        </is>
+      </c>
+      <c r="B97" s="3" t="n"/>
+      <c r="C97" s="3" t="n"/>
+      <c r="D97" s="3" t="n"/>
+      <c r="E97" s="3" t="n"/>
+      <c r="F97" s="3" t="n"/>
+      <c r="G97" s="3" t="n"/>
+      <c r="H97" s="3" t="n"/>
+      <c r="I97" s="3" t="n"/>
+      <c r="J97" s="3" t="n"/>
+      <c r="K97" s="3" t="n"/>
+    </row>
+    <row r="99">
+      <c r="A99" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ITEM c) Fluxo ótimo (De → Para) e quantidades por tipo de veículo:
+=== Minivan (multiplicador de custo: ×1.15) ===
+  • Porto 1 → Distrib. 1: 325 veículos  (custo unit. ajustado: $115.00, custo total arco: $37,375.00)
+  • Porto 2 → Distrib. 2: 430 veículos  (custo unit. ajustado: $138.00, custo total arco: $59,340.00)
+  • Distrib. 1 → Revenda 3: 47 veículos  (custo unit. ajustado: $184.00, custo total arco: $8,648.00)
+  • Distrib. 1 → Revenda 2: 278 veículos  (custo unit. ajustado: $195.50, custo total arco: $54,349.00)
+  • Distrib. 2 → Revenda 3: 430 veículos  (custo unit. ajustado: $161.00, custo total arco: $69,230.00)
+=== Esportivo (multiplicador de custo: ×0.90) ===
+  • Porto 1 → Distrib. 1: 450 veículos  (custo unit. ajustado: $90.00, custo total arco: $40,500.00)
+  • Porto 2 → Distrib. 2: 300 veículos  (custo unit. ajustado: $108.00, custo total arco: $32,400.00)
+  • Distrib. 1 → Revenda 2: 450 veículos  (custo unit. ajustado: $153.00, custo total arco: $68,850.00)
+  • Distrib. 2 → Revenda 3: 227 veículos  (custo unit. ajustado: $126.00, custo total arco: $28,602.00)
+  • Distrib. 2 → Revenda 2: 73 veículos  (custo unit. ajustado: $144.00, custo total arco: $10,512.00)
 </t>
         </is>
       </c>
     </row>
-    <row r="79"/>
-    <row r="80"/>
-    <row r="81"/>
-    <row r="82"/>
-    <row r="83"/>
-    <row r="84"/>
-    <row r="85"/>
-    <row r="86"/>
-    <row r="87"/>
-    <row r="88"/>
-    <row r="89"/>
-    <row r="90"/>
-    <row r="91"/>
-    <row r="92"/>
-    <row r="93"/>
-    <row r="95">
-      <c r="A95" s="28" t="inlineStr">
-        <is>
-          <t>ITEM d) O valor do custo mínimo total dessa operação é: $409,806.00</t>
-        </is>
-      </c>
-    </row>
-    <row r="96"/>
-    <row r="98">
-      <c r="A98" s="2" t="inlineStr">
+    <row r="100"/>
+    <row r="101"/>
+    <row r="102"/>
+    <row r="103"/>
+    <row r="104"/>
+    <row r="105"/>
+    <row r="106"/>
+    <row r="107"/>
+    <row r="108"/>
+    <row r="109"/>
+    <row r="110"/>
+    <row r="111"/>
+    <row r="112"/>
+    <row r="113"/>
+    <row r="114"/>
+    <row r="115"/>
+    <row r="117">
+      <c r="A117" s="32" t="inlineStr">
+        <is>
+          <t>ITEM d) O custo mínimo total dessa operação é: $409,806.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="118"/>
+    <row r="120">
+      <c r="A120" s="2" t="inlineStr">
         <is>
           <t>7. ANÁLISE DE SENSIBILIDADE — Item e)</t>
         </is>
       </c>
-      <c r="B98" s="3" t="n"/>
-      <c r="C98" s="3" t="n"/>
-      <c r="D98" s="3" t="n"/>
-      <c r="E98" s="3" t="n"/>
-      <c r="F98" s="3" t="n"/>
-      <c r="G98" s="3" t="n"/>
-      <c r="H98" s="3" t="n"/>
-      <c r="I98" s="3" t="n"/>
-      <c r="J98" s="3" t="n"/>
-      <c r="K98" s="3" t="n"/>
-    </row>
-    <row r="100">
-      <c r="A100" s="4" t="inlineStr">
-        <is>
-          <t>Variação do custo total conforme capacidade máxima por arco (500 a 1500, intervalos de 100)</t>
-        </is>
-      </c>
-    </row>
-    <row r="101">
-      <c r="A101" s="5" t="inlineStr">
+      <c r="B120" s="3" t="n"/>
+      <c r="C120" s="3" t="n"/>
+      <c r="D120" s="3" t="n"/>
+      <c r="E120" s="3" t="n"/>
+      <c r="F120" s="3" t="n"/>
+      <c r="G120" s="3" t="n"/>
+      <c r="H120" s="3" t="n"/>
+      <c r="I120" s="3" t="n"/>
+      <c r="J120" s="3" t="n"/>
+      <c r="K120" s="3" t="n"/>
+    </row>
+    <row r="122">
+      <c r="A122" s="4" t="inlineStr">
+        <is>
+          <t>Como o custo total varia quando a capacidade máxima de cada arco vai de 500 a 1500 veículos:</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="5" t="inlineStr">
         <is>
           <t>Capacidade Máx/Arco</t>
         </is>
       </c>
-      <c r="B101" s="5" t="inlineStr">
-        <is>
-          <t>Custo Total</t>
-        </is>
-      </c>
-      <c r="C101" s="5" t="inlineStr">
+      <c r="B123" s="5" t="inlineStr">
+        <is>
+          <t>Custo Total ($)</t>
+        </is>
+      </c>
+      <c r="C123" s="5" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-    </row>
-    <row r="102">
-      <c r="A102" s="8" t="n">
+      <c r="D123" s="5" t="inlineStr">
+        <is>
+          <t>Variação vs Sem Limite</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="8" t="n">
         <v>500</v>
       </c>
-      <c r="B102" s="29" t="n">
+      <c r="B124" s="33" t="n">
         <v>420309</v>
       </c>
-      <c r="C102" s="19" t="inlineStr">
+      <c r="C124" s="18" t="inlineStr">
         <is>
           <t>Viável</t>
         </is>
       </c>
-    </row>
-    <row r="103">
-      <c r="A103" s="8" t="n">
+      <c r="D124" s="34">
+        <f>(B124-409806.0)/409806.0</f>
+        <v/>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="8" t="n">
         <v>600</v>
       </c>
-      <c r="B103" s="29" t="n">
+      <c r="B125" s="33" t="n">
         <v>415809</v>
       </c>
-      <c r="C103" s="19" t="inlineStr">
+      <c r="C125" s="18" t="inlineStr">
         <is>
           <t>Viável</t>
         </is>
       </c>
-    </row>
-    <row r="104">
-      <c r="A104" s="8" t="n">
+      <c r="D125" s="34">
+        <f>(B125-409806.0)/409806.0</f>
+        <v/>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="8" t="n">
         <v>700</v>
       </c>
-      <c r="B104" s="29" t="n">
+      <c r="B126" s="33" t="n">
         <v>411416.5</v>
       </c>
-      <c r="C104" s="19" t="inlineStr">
+      <c r="C126" s="18" t="inlineStr">
         <is>
           <t>Viável</t>
         </is>
       </c>
-    </row>
-    <row r="105">
-      <c r="A105" s="8" t="n">
+      <c r="D126" s="34">
+        <f>(B126-409806.0)/409806.0</f>
+        <v/>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="8" t="n">
         <v>800</v>
       </c>
-      <c r="B105" s="29" t="n">
+      <c r="B127" s="33" t="n">
         <v>409806</v>
       </c>
-      <c r="C105" s="19" t="inlineStr">
+      <c r="C127" s="18" t="inlineStr">
         <is>
           <t>Viável</t>
         </is>
       </c>
-    </row>
-    <row r="106">
-      <c r="A106" s="8" t="n">
+      <c r="D127" s="34">
+        <f>(B127-409806.0)/409806.0</f>
+        <v/>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="8" t="n">
         <v>900</v>
       </c>
-      <c r="B106" s="29" t="n">
+      <c r="B128" s="33" t="n">
         <v>409806</v>
       </c>
-      <c r="C106" s="19" t="inlineStr">
+      <c r="C128" s="18" t="inlineStr">
         <is>
           <t>Viável</t>
         </is>
       </c>
-    </row>
-    <row r="107">
-      <c r="A107" s="8" t="n">
+      <c r="D128" s="34">
+        <f>(B128-409806.0)/409806.0</f>
+        <v/>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="8" t="n">
         <v>1000</v>
       </c>
-      <c r="B107" s="29" t="n">
+      <c r="B129" s="33" t="n">
         <v>409806</v>
       </c>
-      <c r="C107" s="19" t="inlineStr">
+      <c r="C129" s="18" t="inlineStr">
         <is>
           <t>Viável</t>
         </is>
       </c>
-    </row>
-    <row r="108">
-      <c r="A108" s="8" t="n">
+      <c r="D129" s="34">
+        <f>(B129-409806.0)/409806.0</f>
+        <v/>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="8" t="n">
         <v>1100</v>
       </c>
-      <c r="B108" s="29" t="n">
+      <c r="B130" s="33" t="n">
         <v>409806</v>
       </c>
-      <c r="C108" s="19" t="inlineStr">
+      <c r="C130" s="18" t="inlineStr">
         <is>
           <t>Viável</t>
         </is>
       </c>
-    </row>
-    <row r="109">
-      <c r="A109" s="8" t="n">
+      <c r="D130" s="34">
+        <f>(B130-409806.0)/409806.0</f>
+        <v/>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="8" t="n">
         <v>1200</v>
       </c>
-      <c r="B109" s="29" t="n">
+      <c r="B131" s="33" t="n">
         <v>409806</v>
       </c>
-      <c r="C109" s="19" t="inlineStr">
+      <c r="C131" s="18" t="inlineStr">
         <is>
           <t>Viável</t>
         </is>
       </c>
-    </row>
-    <row r="110">
-      <c r="A110" s="8" t="n">
+      <c r="D131" s="34">
+        <f>(B131-409806.0)/409806.0</f>
+        <v/>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="8" t="n">
         <v>1300</v>
       </c>
-      <c r="B110" s="29" t="n">
+      <c r="B132" s="33" t="n">
         <v>409806</v>
       </c>
-      <c r="C110" s="19" t="inlineStr">
+      <c r="C132" s="18" t="inlineStr">
         <is>
           <t>Viável</t>
         </is>
       </c>
-    </row>
-    <row r="111">
-      <c r="A111" s="8" t="n">
+      <c r="D132" s="34">
+        <f>(B132-409806.0)/409806.0</f>
+        <v/>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="8" t="n">
         <v>1400</v>
       </c>
-      <c r="B111" s="29" t="n">
+      <c r="B133" s="33" t="n">
         <v>409806</v>
       </c>
-      <c r="C111" s="19" t="inlineStr">
+      <c r="C133" s="18" t="inlineStr">
         <is>
           <t>Viável</t>
         </is>
       </c>
-    </row>
-    <row r="112">
-      <c r="A112" s="8" t="n">
+      <c r="D133" s="34">
+        <f>(B133-409806.0)/409806.0</f>
+        <v/>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="8" t="n">
         <v>1500</v>
       </c>
-      <c r="B112" s="29" t="n">
+      <c r="B134" s="33" t="n">
         <v>409806</v>
       </c>
-      <c r="C112" s="19" t="inlineStr">
+      <c r="C134" s="18" t="inlineStr">
         <is>
           <t>Viável</t>
         </is>
       </c>
-    </row>
-    <row r="114">
-      <c r="A114" s="25" t="inlineStr">
-        <is>
-          <t>ITEM e) Análise de Sensibilidade:
-Capacidade Máx/Arco → Custo Total:
-    500 veículos → $  420,309.00
-    600 veículos → $  415,809.00
-    700 veículos → $  411,416.50
-    800 veículos → $  409,806.00
-    900 veículos → $  409,806.00
-   1000 veículos → $  409,806.00
-   1100 veículos → $  409,806.00
-   1200 veículos → $  409,806.00
-   1300 veículos → $  409,806.00
-   1400 veículos → $  409,806.00
-   1500 veículos → $  409,806.00
-O custo mínimo de $409,806.00 é atingido a partir da capacidade de 800 veículos/arco.
-Abaixo desse valor, as restrições de capacidade forçam rotas mais caras ou tornam o problema inviável.</t>
-        </is>
-      </c>
-    </row>
-    <row r="115"/>
-    <row r="116"/>
-    <row r="117"/>
-    <row r="118"/>
-    <row r="119"/>
-    <row r="120"/>
-    <row r="121"/>
-    <row r="122"/>
-    <row r="123"/>
-    <row r="124"/>
-    <row r="125"/>
-    <row r="126"/>
-    <row r="127"/>
-    <row r="128"/>
+      <c r="D134" s="34">
+        <f>(B134-409806.0)/409806.0</f>
+        <v/>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="25" t="inlineStr">
+        <is>
+          <t>ITEM e) Análise de Sensibilidade — Resposta por extenso:
+Capacidade Máx/Arco  →  Custo Total
+    500 veículos  →  $  420,309.00  (diferença: $+10,503.00)
+    600 veículos  →  $  415,809.00  (diferença: $ +6,003.00)
+    700 veículos  →  $  411,416.50  (diferença: $ +1,610.50)
+    800 veículos  →  $  409,806.00  (diferença: $     +0.00)
+    900 veículos  →  $  409,806.00  (diferença: $     +0.00)
+   1000 veículos  →  $  409,806.00  (diferença: $     +0.00)
+   1100 veículos  →  $  409,806.00  (diferença: $     +0.00)
+   1200 veículos  →  $  409,806.00  (diferença: $     +0.00)
+   1300 veículos  →  $  409,806.00  (diferença: $     +0.00)
+   1400 veículos  →  $  409,806.00  (diferença: $     +0.00)
+   1500 veículos  →  $  409,806.00  (diferença: $     +0.00)
+Conclusão: O custo mínimo de $409,806.00 (igual ao caso sem restrição de capacidade)
+é atingido a partir de 800 veículos/arco. Abaixo desse valor, as restrições de
+capacidade forçam o uso de rotas mais caras, elevando o custo total.</t>
+        </is>
+      </c>
+    </row>
+    <row r="137"/>
+    <row r="138"/>
+    <row r="139"/>
+    <row r="140"/>
+    <row r="141"/>
+    <row r="142"/>
+    <row r="143"/>
+    <row r="144"/>
+    <row r="145"/>
+    <row r="146"/>
+    <row r="147"/>
+    <row r="148"/>
+    <row r="149"/>
+    <row r="150"/>
+    <row r="151"/>
+    <row r="152"/>
   </sheetData>
-  <mergeCells count="12">
-    <mergeCell ref="A114:K128"/>
+  <mergeCells count="20">
     <mergeCell ref="A48:K48"/>
+    <mergeCell ref="B74:K74"/>
+    <mergeCell ref="A99:K115"/>
+    <mergeCell ref="B95:K95"/>
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A136:K152"/>
+    <mergeCell ref="B94:K94"/>
+    <mergeCell ref="A69:K69"/>
+    <mergeCell ref="B75:K75"/>
+    <mergeCell ref="A122:F122"/>
+    <mergeCell ref="B72:K72"/>
+    <mergeCell ref="A120:K120"/>
+    <mergeCell ref="B71:K71"/>
     <mergeCell ref="A3:K3"/>
-    <mergeCell ref="A100:F100"/>
-    <mergeCell ref="A95:K96"/>
+    <mergeCell ref="B93:K93"/>
+    <mergeCell ref="A117:K118"/>
+    <mergeCell ref="A97:K97"/>
     <mergeCell ref="A52:K52"/>
-    <mergeCell ref="A78:K93"/>
-    <mergeCell ref="A98:K98"/>
-    <mergeCell ref="A76:K76"/>
-    <mergeCell ref="A68:K68"/>
-    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="B73:K73"/>
     <mergeCell ref="A31:K31"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>